<commit_message>
Save: workbooks, R1 recap draft, golf icons, processed_files state
</commit_message>
<xml_diff>
--- a/Score Calculator.xlsx
+++ b/Score Calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imicompanies-my.sharepoint.com/personal/ehigh_iengtobuild_com/Documents/Documents/Golf League/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="8_{A2D2493B-942A-431B-BFE9-D343A07FD7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D576A356-9504-47F7-A006-ADCF5FF2621E}"/>
+  <xr:revisionPtr revIDLastSave="88" documentId="8_{A2D2493B-942A-431B-BFE9-D343A07FD7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03A718E0-DC5D-45F6-AC24-BE50171BB2CB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A94AAD03-8B68-4D25-ACDC-485563D823F1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A94AAD03-8B68-4D25-ACDC-485563D823F1}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculator" sheetId="1" r:id="rId1"/>
@@ -581,6 +581,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -604,12 +610,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -664,11 +664,11 @@
       <sheetName val="Oct 14 - 25th"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
       <sheetData sheetId="5">
         <row r="15">
           <cell r="D15">
@@ -715,11 +715,6 @@
             <v>30</v>
           </cell>
         </row>
-        <row r="24">
-          <cell r="D24">
-            <v>36</v>
-          </cell>
-        </row>
         <row r="25">
           <cell r="D25">
             <v>36</v>
@@ -746,14 +741,14 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1077,43 +1072,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C7E9C1E-B4F8-42BE-ADD6-CFDCDE6729D4}">
   <dimension ref="B1:BG29"/>
-  <sheetFormatPr defaultColWidth="9.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.5703125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
-    <col min="3" max="8" width="9.85546875" style="2" customWidth="1"/>
-    <col min="9" max="9" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="10.5703125" style="2" customWidth="1"/>
-    <col min="12" max="13" width="10.85546875" style="2" customWidth="1"/>
-    <col min="14" max="14" width="5.7109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="2.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" style="2" customWidth="1"/>
+    <col min="3" max="8" width="9.88671875" style="2" customWidth="1"/>
+    <col min="9" max="9" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="10.5546875" style="2" customWidth="1"/>
+    <col min="12" max="13" width="10.88671875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="5.6640625" style="2" customWidth="1"/>
     <col min="15" max="15" width="11" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="4.5703125" style="2" customWidth="1"/>
+    <col min="16" max="16" width="16.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="4.5546875" style="2" customWidth="1"/>
     <col min="20" max="20" width="11" style="2" bestFit="1" customWidth="1"/>
     <col min="21" max="29" width="4" style="2" customWidth="1"/>
-    <col min="30" max="30" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="10.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="31" max="39" width="4" style="2" customWidth="1"/>
     <col min="40" max="40" width="11" style="2" bestFit="1" customWidth="1"/>
     <col min="41" max="49" width="4" style="2" customWidth="1"/>
-    <col min="50" max="50" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="10.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="51" max="59" width="4" style="2" customWidth="1"/>
-    <col min="60" max="65" width="9.85546875" style="2" customWidth="1"/>
-    <col min="66" max="16384" width="9.85546875" style="2"/>
+    <col min="60" max="65" width="9.88671875" style="2" customWidth="1"/>
+    <col min="66" max="16384" width="9.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J1" s="39" t="s">
+      <c r="J1" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
     </row>
-    <row r="2" spans="2:59" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:59" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
@@ -1133,21 +1128,21 @@
         <v>7</v>
       </c>
       <c r="I2" s="5"/>
-      <c r="J2" s="41" t="str">
+      <c r="J2" s="43" t="str">
         <f>B8</f>
-        <v>Rob Bass</v>
-      </c>
-      <c r="K2" s="42"/>
-      <c r="L2" s="43" t="str">
+        <v>Megan Serian</v>
+      </c>
+      <c r="K2" s="44"/>
+      <c r="L2" s="45" t="str">
         <f>B17</f>
-        <v>Carson Bass</v>
-      </c>
-      <c r="M2" s="42"/>
+        <v>Nick Coglianese</v>
+      </c>
+      <c r="M2" s="44"/>
     </row>
-    <row r="3" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="44" t="str">
+    <row r="3" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="46" t="str">
         <f>J2</f>
-        <v>Rob Bass</v>
+        <v>Megan Serian</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>8</v>
@@ -1162,121 +1157,121 @@
       </c>
       <c r="F3" s="7">
         <f>SUM(I15:K15)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" s="7">
         <f>SUM(C15:K15)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H3" s="7">
         <f>SUM(C14:K14)</f>
-        <v>43</v>
-      </c>
-      <c r="J3" s="46">
+        <v>50</v>
+      </c>
+      <c r="J3" s="48">
         <f>SUM(D4:H4)</f>
+        <v>7</v>
+      </c>
+      <c r="K3" s="49"/>
+      <c r="L3" s="53">
+        <f>SUM(D6:H6)</f>
         <v>1</v>
       </c>
-      <c r="K3" s="47"/>
-      <c r="L3" s="51">
-        <f>SUM(D6:H6)</f>
-        <v>7</v>
-      </c>
-      <c r="M3" s="47"/>
+      <c r="M3" s="49"/>
     </row>
-    <row r="4" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="45"/>
+    <row r="4" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="47"/>
       <c r="C4" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="9">
         <f>IF(D3&gt;D5,2,IF(D3=D5,1,0))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E4" s="9">
         <f>IF(E3&gt;E5,2,IF(E3=E5,1,0))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" s="9">
         <f>IF(F3&gt;F5,2,IF(F3=F5,1,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" s="9">
         <f>IF(G3&gt;G5,1,IF(G3=G5,0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="9">
         <f>IF(H3&lt;H5,1,IF(H3=H5,0.5,0))</f>
-        <v>0</v>
-      </c>
-      <c r="J4" s="48"/>
-      <c r="K4" s="49"/>
-      <c r="L4" s="52"/>
-      <c r="M4" s="49"/>
+        <v>1</v>
+      </c>
+      <c r="J4" s="50"/>
+      <c r="K4" s="51"/>
+      <c r="L4" s="40"/>
+      <c r="M4" s="51"/>
     </row>
-    <row r="5" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="44" t="str">
+    <row r="5" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="46" t="str">
         <f>L2</f>
-        <v>Carson Bass</v>
+        <v>Nick Coglianese</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="11">
         <f>SUM(C24:E24)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E5" s="11">
         <f>SUM(F24:H24)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="11">
         <f>SUM(I24:K24)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5" s="11">
         <f>SUM(C24:K24)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H5" s="11">
         <f>SUM(C23:K23)</f>
-        <v>38</v>
-      </c>
-      <c r="J5" s="45"/>
-      <c r="K5" s="50"/>
-      <c r="L5" s="40"/>
-      <c r="M5" s="50"/>
+        <v>53</v>
+      </c>
+      <c r="J5" s="47"/>
+      <c r="K5" s="52"/>
+      <c r="L5" s="42"/>
+      <c r="M5" s="52"/>
     </row>
-    <row r="6" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="45"/>
+    <row r="6" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="47"/>
       <c r="C6" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D6" s="9">
         <f>IF(D5&gt;D3,2,IF(D5=D3,1,0))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E6" s="9">
         <f>IF(E5&gt;E3,2,IF(E5=E3,1,0))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="9">
         <f>IF(F5&gt;F3,2,IF(F5=F3,1,0))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" s="9">
         <f>IF(G5&gt;G3,1,IF(G5=G3,0.5,0))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" s="9">
         <f>IF(H5&lt;H3,1,IF(H5=H3,0.5,0))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" s="12"/>
       <c r="K6" s="12"/>
       <c r="L6" s="12"/>
       <c r="M6" s="12"/>
     </row>
-    <row r="7" spans="2:59" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:59" x14ac:dyDescent="0.25">
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
       <c r="E7" s="12"/>
@@ -1287,68 +1282,68 @@
       <c r="J7" s="12"/>
       <c r="K7" s="12"/>
       <c r="L7" s="12"/>
-      <c r="T7" s="53" t="s">
-        <v>2</v>
-      </c>
-      <c r="U7" s="52"/>
-      <c r="V7" s="52"/>
-      <c r="W7" s="52"/>
-      <c r="X7" s="52"/>
-      <c r="Y7" s="52"/>
-      <c r="Z7" s="52"/>
-      <c r="AA7" s="52"/>
-      <c r="AB7" s="52"/>
-      <c r="AC7" s="52"/>
-      <c r="AD7" s="52"/>
-      <c r="AE7" s="52"/>
-      <c r="AF7" s="52"/>
-      <c r="AG7" s="52"/>
-      <c r="AH7" s="52"/>
-      <c r="AI7" s="52"/>
-      <c r="AJ7" s="52"/>
-      <c r="AK7" s="52"/>
-      <c r="AL7" s="52"/>
-      <c r="AM7" s="52"/>
-      <c r="AN7" s="53" t="s">
+      <c r="T7" s="39" t="s">
+        <v>2</v>
+      </c>
+      <c r="U7" s="40"/>
+      <c r="V7" s="40"/>
+      <c r="W7" s="40"/>
+      <c r="X7" s="40"/>
+      <c r="Y7" s="40"/>
+      <c r="Z7" s="40"/>
+      <c r="AA7" s="40"/>
+      <c r="AB7" s="40"/>
+      <c r="AC7" s="40"/>
+      <c r="AD7" s="40"/>
+      <c r="AE7" s="40"/>
+      <c r="AF7" s="40"/>
+      <c r="AG7" s="40"/>
+      <c r="AH7" s="40"/>
+      <c r="AI7" s="40"/>
+      <c r="AJ7" s="40"/>
+      <c r="AK7" s="40"/>
+      <c r="AL7" s="40"/>
+      <c r="AM7" s="40"/>
+      <c r="AN7" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="AO7" s="52"/>
-      <c r="AP7" s="52"/>
-      <c r="AQ7" s="52"/>
-      <c r="AR7" s="52"/>
-      <c r="AS7" s="52"/>
-      <c r="AT7" s="52"/>
-      <c r="AU7" s="52"/>
-      <c r="AV7" s="52"/>
-      <c r="AW7" s="52"/>
-      <c r="AX7" s="52"/>
-      <c r="AY7" s="52"/>
-      <c r="AZ7" s="52"/>
-      <c r="BA7" s="52"/>
-      <c r="BB7" s="52"/>
-      <c r="BC7" s="52"/>
-      <c r="BD7" s="52"/>
-      <c r="BE7" s="52"/>
-      <c r="BF7" s="52"/>
-      <c r="BG7" s="52"/>
+      <c r="AO7" s="40"/>
+      <c r="AP7" s="40"/>
+      <c r="AQ7" s="40"/>
+      <c r="AR7" s="40"/>
+      <c r="AS7" s="40"/>
+      <c r="AT7" s="40"/>
+      <c r="AU7" s="40"/>
+      <c r="AV7" s="40"/>
+      <c r="AW7" s="40"/>
+      <c r="AX7" s="40"/>
+      <c r="AY7" s="40"/>
+      <c r="AZ7" s="40"/>
+      <c r="BA7" s="40"/>
+      <c r="BB7" s="40"/>
+      <c r="BC7" s="40"/>
+      <c r="BD7" s="40"/>
+      <c r="BE7" s="40"/>
+      <c r="BF7" s="40"/>
+      <c r="BG7" s="40"/>
     </row>
-    <row r="8" spans="2:59" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:59" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="13" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="C8" s="14" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="12">
         <f>_xlfn.XLOOKUP(B8,$P$9:$P$23,$Q$9:$Q$23)</f>
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="12" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="H8" s="12"/>
       <c r="I8" s="12" t="s">
@@ -1371,57 +1366,57 @@
       <c r="T8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="U8" s="53" t="s">
+      <c r="U8" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="V8" s="52"/>
-      <c r="W8" s="52"/>
-      <c r="X8" s="52"/>
-      <c r="Y8" s="52"/>
-      <c r="Z8" s="52"/>
-      <c r="AA8" s="52"/>
-      <c r="AB8" s="52"/>
-      <c r="AC8" s="52"/>
-      <c r="AD8" s="53" t="s">
+      <c r="V8" s="40"/>
+      <c r="W8" s="40"/>
+      <c r="X8" s="40"/>
+      <c r="Y8" s="40"/>
+      <c r="Z8" s="40"/>
+      <c r="AA8" s="40"/>
+      <c r="AB8" s="40"/>
+      <c r="AC8" s="40"/>
+      <c r="AD8" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="AE8" s="52"/>
-      <c r="AF8" s="52"/>
-      <c r="AG8" s="52"/>
-      <c r="AH8" s="52"/>
-      <c r="AI8" s="52"/>
-      <c r="AJ8" s="52"/>
-      <c r="AK8" s="52"/>
-      <c r="AL8" s="52"/>
-      <c r="AM8" s="52"/>
+      <c r="AE8" s="40"/>
+      <c r="AF8" s="40"/>
+      <c r="AG8" s="40"/>
+      <c r="AH8" s="40"/>
+      <c r="AI8" s="40"/>
+      <c r="AJ8" s="40"/>
+      <c r="AK8" s="40"/>
+      <c r="AL8" s="40"/>
+      <c r="AM8" s="40"/>
       <c r="AN8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="AO8" s="53" t="s">
+      <c r="AO8" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="AP8" s="52"/>
-      <c r="AQ8" s="52"/>
-      <c r="AR8" s="52"/>
-      <c r="AS8" s="52"/>
-      <c r="AT8" s="52"/>
-      <c r="AU8" s="52"/>
-      <c r="AV8" s="52"/>
-      <c r="AW8" s="52"/>
-      <c r="AX8" s="53" t="s">
+      <c r="AP8" s="40"/>
+      <c r="AQ8" s="40"/>
+      <c r="AR8" s="40"/>
+      <c r="AS8" s="40"/>
+      <c r="AT8" s="40"/>
+      <c r="AU8" s="40"/>
+      <c r="AV8" s="40"/>
+      <c r="AW8" s="40"/>
+      <c r="AX8" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="AY8" s="52"/>
-      <c r="AZ8" s="52"/>
-      <c r="BA8" s="52"/>
-      <c r="BB8" s="52"/>
-      <c r="BC8" s="52"/>
-      <c r="BD8" s="52"/>
-      <c r="BE8" s="52"/>
-      <c r="BF8" s="52"/>
-      <c r="BG8" s="52"/>
+      <c r="AY8" s="40"/>
+      <c r="AZ8" s="40"/>
+      <c r="BA8" s="40"/>
+      <c r="BB8" s="40"/>
+      <c r="BC8" s="40"/>
+      <c r="BD8" s="40"/>
+      <c r="BE8" s="40"/>
+      <c r="BF8" s="40"/>
+      <c r="BG8" s="40"/>
     </row>
-    <row r="9" spans="2:59" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:59" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="18" t="s">
         <v>22</v>
       </c>
@@ -1584,7 +1579,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="2:59" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:59" x14ac:dyDescent="0.3">
       <c r="B10" s="25" t="s">
         <v>24</v>
       </c>
@@ -1840,7 +1835,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="2:59" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:59" x14ac:dyDescent="0.3">
       <c r="B11" s="25" t="s">
         <v>28</v>
       </c>
@@ -1855,7 +1850,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D11" s="12">
         <f t="array" ref="D11">IF($B$2="Skybrook",
@@ -1868,7 +1863,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E11" s="26">
         <f t="array" ref="E11">IF($B$2="Skybrook",
@@ -1894,7 +1889,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="G11" s="12">
         <f t="array" ref="G11">IF($B$2="Skybrook",
@@ -1920,7 +1915,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I11" s="27">
         <f t="array" ref="I11">IF($B$2="Skybrook",
@@ -1933,7 +1928,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="J11" s="12">
         <f t="array" ref="J11">IF($B$2="Skybrook",
@@ -1946,7 +1941,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="K11" s="26">
         <f t="array" ref="K11">IF($B$2="Skybrook",
@@ -2094,44 +2089,44 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="2:59" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:59" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="28" t="s">
         <v>31</v>
       </c>
       <c r="C12" s="29">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D12" s="30">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E12" s="31">
+        <v>8</v>
+      </c>
+      <c r="F12" s="29">
+        <v>9</v>
+      </c>
+      <c r="G12" s="30">
+        <v>8</v>
+      </c>
+      <c r="H12" s="31">
+        <v>8</v>
+      </c>
+      <c r="I12" s="29">
         <v>6</v>
       </c>
-      <c r="F12" s="29">
-        <v>7</v>
-      </c>
-      <c r="G12" s="30">
-        <v>7</v>
-      </c>
-      <c r="H12" s="31">
-        <v>6</v>
-      </c>
-      <c r="I12" s="29">
-        <v>4</v>
-      </c>
       <c r="J12" s="30">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="K12" s="31">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L12" s="12">
         <f>SUM(C12:K12)</f>
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="M12" s="32">
         <f>SUM(C12:K12)-SUM(C$10:K$10)</f>
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="O12" s="22">
         <v>4</v>
@@ -2264,45 +2259,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="2:59" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:59" x14ac:dyDescent="0.3">
       <c r="B13" s="25" t="s">
         <v>34</v>
       </c>
       <c r="C13" s="27">
         <f t="shared" ref="C13:K13" si="0">INT($D$8/18)+IF(C11&lt;=MOD($D$8,18),1,0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" s="12">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" s="26">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="27">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G13" s="12">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H13" s="26">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I13" s="27">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J13" s="12">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="26">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L13" s="32"/>
       <c r="O13" s="22">
@@ -2316,7 +2311,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="2:59" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:59" x14ac:dyDescent="0.3">
       <c r="B14" s="25" t="s">
         <v>36</v>
       </c>
@@ -2326,15 +2321,15 @@
       </c>
       <c r="D14" s="12">
         <f t="shared" ref="D14:K14" si="1">D12-INT($D$8/18)-IF(D11&lt;=MOD($D$8,18),1,0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14" s="26">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F14" s="27">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G14" s="12">
         <f t="shared" si="1"/>
@@ -2342,7 +2337,7 @@
       </c>
       <c r="H14" s="26">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I14" s="27">
         <f t="shared" si="1"/>
@@ -2350,7 +2345,7 @@
       </c>
       <c r="J14" s="12">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K14" s="26">
         <f t="shared" si="1"/>
@@ -2358,11 +2353,11 @@
       </c>
       <c r="L14" s="34">
         <f>SUM(C14:K14)</f>
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="M14" s="32">
         <f>SUM(C14:K14)-SUM(C$10:K$10)</f>
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="O14" s="22">
         <v>6</v>
@@ -2375,17 +2370,17 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="35" t="s">
         <v>38</v>
       </c>
       <c r="C15" s="36">
         <f t="shared" ref="C15:K15" si="2">IF(C14&lt;C23,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" s="37">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="38">
         <f t="shared" si="2"/>
@@ -2393,7 +2388,7 @@
       </c>
       <c r="F15" s="36">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" s="37">
         <f t="shared" si="2"/>
@@ -2401,7 +2396,7 @@
       </c>
       <c r="H15" s="38">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15" s="36">
         <f t="shared" si="2"/>
@@ -2409,7 +2404,7 @@
       </c>
       <c r="J15" s="37">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" s="38">
         <f t="shared" si="2"/>
@@ -2428,7 +2423,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="2:59" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:59" x14ac:dyDescent="0.3">
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
       <c r="E16" s="12"/>
@@ -2450,16 +2445,16 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="2:42" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:42" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="13" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="C17" s="14" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="12">
         <f>_xlfn.XLOOKUP(B17,$P$9:$P$23,$Q$9:$Q$23)</f>
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E17" s="12"/>
       <c r="F17" s="12" t="s">
@@ -2489,7 +2484,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="2:42" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:42" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="18" t="s">
         <v>22</v>
       </c>
@@ -2529,11 +2524,10 @@
         <v>42</v>
       </c>
       <c r="Q18" s="24">
-        <f>[1]Schedule!D24</f>
-        <v>36</v>
+        <v>20</v>
       </c>
     </row>
-    <row r="19" spans="2:42" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:42" x14ac:dyDescent="0.3">
       <c r="B19" s="25" t="s">
         <v>24</v>
       </c>
@@ -2670,7 +2664,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="2:42" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:42" x14ac:dyDescent="0.3">
       <c r="B20" s="25" t="s">
         <v>28</v>
       </c>
@@ -2803,44 +2797,44 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="2:42" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:42" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="28" t="s">
         <v>31</v>
       </c>
       <c r="C21" s="29">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D21" s="30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E21" s="31">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F21" s="29">
+        <v>10</v>
+      </c>
+      <c r="G21" s="30">
+        <v>8</v>
+      </c>
+      <c r="H21" s="31">
+        <v>8</v>
+      </c>
+      <c r="I21" s="29">
         <v>6</v>
       </c>
-      <c r="G21" s="30">
-        <v>7</v>
-      </c>
-      <c r="H21" s="31">
-        <v>7</v>
-      </c>
-      <c r="I21" s="29">
-        <v>4</v>
-      </c>
       <c r="J21" s="30">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K21" s="31">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L21" s="12">
         <f>SUM(C21:K21)</f>
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="M21" s="32">
         <f>SUM(C21:K21)-SUM(C$10:K$10)</f>
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="O21" s="22">
         <v>13</v>
@@ -2853,41 +2847,41 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="2:42" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:42" x14ac:dyDescent="0.3">
       <c r="B22" s="25" t="s">
         <v>34</v>
       </c>
       <c r="C22" s="27">
         <f t="shared" ref="C22:K22" si="3">INT($D$17/18)+IF(C20&lt;=MOD($D$17,18),1,0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" s="12">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22" s="26">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" s="27">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22" s="12">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H22" s="26">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I22" s="27">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J22" s="12">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K22" s="26">
         <f t="shared" si="3"/>
@@ -2905,13 +2899,13 @@
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="2:42" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:42" x14ac:dyDescent="0.3">
       <c r="B23" s="25" t="s">
         <v>36</v>
       </c>
       <c r="C23" s="27">
         <f t="shared" ref="C23:K23" si="4">C21-C22</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D23" s="12">
         <f t="shared" si="4"/>
@@ -2919,11 +2913,11 @@
       </c>
       <c r="E23" s="26">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F23" s="27">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G23" s="12">
         <f t="shared" si="4"/>
@@ -2935,23 +2929,23 @@
       </c>
       <c r="I23" s="27">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J23" s="12">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K23" s="26">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L23" s="34">
         <f>SUM(C23:K23)</f>
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="M23" s="32">
         <f>SUM(C23:K23)-SUM(C$10:K$10)</f>
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="O23" s="22">
         <v>15</v>
@@ -2964,13 +2958,13 @@
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="2:42" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:42" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="35" t="s">
         <v>38</v>
       </c>
       <c r="C24" s="36">
         <f t="shared" ref="C24:K24" si="5">IF(C23&lt;C14,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D24" s="37">
         <f t="shared" si="5"/>
@@ -2978,11 +2972,11 @@
       </c>
       <c r="E24" s="38">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F24" s="36">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" s="37">
         <f t="shared" si="5"/>
@@ -2994,7 +2988,7 @@
       </c>
       <c r="I24" s="36">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" s="37">
         <f t="shared" si="5"/>
@@ -3002,23 +2996,17 @@
       </c>
       <c r="K24" s="38">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L24" s="12"/>
     </row>
-    <row r="29" spans="2:42" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:42" x14ac:dyDescent="0.25">
       <c r="AP29" s="2" t="s">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="T7:AM7"/>
-    <mergeCell ref="AN7:BG7"/>
-    <mergeCell ref="U8:AC8"/>
-    <mergeCell ref="AD8:AM8"/>
-    <mergeCell ref="AO8:AW8"/>
-    <mergeCell ref="AX8:BG8"/>
     <mergeCell ref="J1:M1"/>
     <mergeCell ref="J2:K2"/>
     <mergeCell ref="L2:M2"/>
@@ -3026,6 +3014,12 @@
     <mergeCell ref="J3:K5"/>
     <mergeCell ref="L3:M5"/>
     <mergeCell ref="B5:B6"/>
+    <mergeCell ref="T7:AM7"/>
+    <mergeCell ref="AN7:BG7"/>
+    <mergeCell ref="U8:AC8"/>
+    <mergeCell ref="AD8:AM8"/>
+    <mergeCell ref="AO8:AW8"/>
+    <mergeCell ref="AX8:BG8"/>
   </mergeCells>
   <conditionalFormatting sqref="C15:K15 C24:K24">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
@@ -3053,13 +3047,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9023B9F3-7138-4C94-97BC-0498273A3425}">
   <dimension ref="C2:D5"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
         <v>2</v>
       </c>
@@ -3067,7 +3061,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
         <v>14</v>
       </c>
@@ -3075,7 +3069,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>26</v>
       </c>
@@ -3083,7 +3077,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
         <v>30</v>
       </c>

</xml_diff>

<commit_message>
R4 makeup: Ethan High def. Alex Palmer 7-1
R4 matches now recorded (2 of 7):
- David Maddox 4-4 Nick Coglianese (draw, both NET 43) — prior
- Ethan High def. Alex Palmer 7-1 (NET 42 vs 49) at Highland Creek

Alex's R4 scorecard used his new handicap of 30 (15 strokes/9); R1-R3
remain at 27. Standings: Ethan up to 20 pts (3-0-0), takes seed #2 behind
Curtis Lynn (21); Alex to 11 pts (1-3-0). Bruce overrides re-applied after
processing; currentRound restored to 5 (processor reset it to 4).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Score Calculator.xlsx
+++ b/Score Calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imicompanies-my.sharepoint.com/personal/ehigh_iengtobuild_com/Documents/Documents/Golf League/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="307" documentId="8_{A2D2493B-942A-431B-BFE9-D343A07FD7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94EA9ED9-57C3-42F3-BB2E-A74E3CB3748B}"/>
+  <xr:revisionPtr revIDLastSave="326" documentId="8_{A2D2493B-942A-431B-BFE9-D343A07FD7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4311BA8-53B1-4C04-97E9-1D9104D582C1}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="44370" yWindow="5970" windowWidth="28800" windowHeight="15345" xr2:uid="{A94AAD03-8B68-4D25-ACDC-485563D823F1}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A94AAD03-8B68-4D25-ACDC-485563D823F1}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculator" sheetId="1" r:id="rId1"/>
@@ -702,7 +702,7 @@
         </row>
         <row r="21">
           <cell r="D21">
-            <v>27</v>
+            <v>30</v>
           </cell>
         </row>
         <row r="22">
@@ -1130,51 +1130,51 @@
       <c r="I2" s="5"/>
       <c r="J2" s="41" t="str">
         <f>B8</f>
-        <v>David Maddox</v>
+        <v>Charlotte Hayes</v>
       </c>
       <c r="K2" s="42"/>
       <c r="L2" s="43" t="str">
         <f>B17</f>
-        <v>Nick Coglianese</v>
+        <v>Megan Serian</v>
       </c>
       <c r="M2" s="42"/>
     </row>
     <row r="3" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B3" s="44" t="str">
         <f>J2</f>
-        <v>David Maddox</v>
+        <v>Charlotte Hayes</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="7">
         <f>SUM(C15:E15)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E3" s="7">
         <f>SUM(F15:H15)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="7">
         <f>SUM(I15:K15)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G3" s="7">
         <f>SUM(C15:K15)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H3" s="7">
         <f>SUM(C14:K14)</f>
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="J3" s="46">
         <f>SUM(D4:H4)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K3" s="47"/>
       <c r="L3" s="51">
         <f>SUM(D6:H6)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M3" s="47"/>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="D4" s="9">
         <f>IF(D3&gt;D5,2,IF(D3=D5,1,0))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="9">
         <f>IF(E3&gt;E5,2,IF(E3=E5,1,0))</f>
@@ -1193,15 +1193,15 @@
       </c>
       <c r="F4" s="9">
         <f>IF(F3&gt;F5,2,IF(F3=F5,1,0))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" s="9">
         <f>IF(G3&gt;G5,1,IF(G3=G5,0.5,0))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H4" s="9">
         <f>IF(H3&lt;H5,1,IF(H3=H5,0.5,0))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J4" s="48"/>
       <c r="K4" s="49"/>
@@ -1211,7 +1211,7 @@
     <row r="5" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B5" s="44" t="str">
         <f>L2</f>
-        <v>Nick Coglianese</v>
+        <v>Megan Serian</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>8</v>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="E5" s="11">
         <f>SUM(F24:H24)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="11">
         <f>SUM(I24:K24)</f>
@@ -1230,11 +1230,11 @@
       </c>
       <c r="G5" s="11">
         <f>SUM(C24:K24)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" s="11">
         <f>SUM(C23:K23)</f>
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="J5" s="45"/>
       <c r="K5" s="50"/>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="D6" s="9">
         <f>IF(D5&gt;D3,2,IF(D5=D3,1,0))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="9">
         <f>IF(E5&gt;E3,2,IF(E5=E3,1,0))</f>
@@ -1256,15 +1256,15 @@
       </c>
       <c r="F6" s="9">
         <f>IF(F5&gt;F3,2,IF(F5=F3,1,0))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="9">
         <f>IF(G5&gt;G3,1,IF(G5=G3,0.5,0))</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H6" s="9">
         <f>IF(H5&lt;H3,1,IF(H5=H3,0.5,0))</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J6" s="12"/>
       <c r="K6" s="12"/>
@@ -1329,14 +1329,14 @@
     </row>
     <row r="8" spans="2:59" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C8" s="14" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="12">
         <f>_xlfn.XLOOKUP(B8,$P$9:$P$23,$Q$9:$Q$23)</f>
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="12" t="s">
@@ -2094,19 +2094,19 @@
         <v>31</v>
       </c>
       <c r="C12" s="29">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D12" s="30">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E12" s="31">
+        <v>3</v>
+      </c>
+      <c r="F12" s="29">
         <v>6</v>
       </c>
-      <c r="F12" s="29">
-        <v>8</v>
-      </c>
       <c r="G12" s="30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H12" s="31">
         <v>6</v>
@@ -2118,15 +2118,15 @@
         <v>6</v>
       </c>
       <c r="K12" s="31">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L12" s="12">
         <f>SUM(C12:K12)</f>
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="M12" s="32">
         <f>SUM(C12:K12)-SUM(C$10:K$10)</f>
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="O12" s="22">
         <v>4</v>
@@ -2265,15 +2265,15 @@
       </c>
       <c r="C13" s="27">
         <f t="shared" ref="C13:K13" si="0">INT($D$8/18)+IF(C11&lt;=MOD($D$8,18),1,0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" s="12">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" s="26">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" s="27">
         <f t="shared" si="0"/>
@@ -2281,23 +2281,23 @@
       </c>
       <c r="G13" s="12">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H13" s="26">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I13" s="27">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J13" s="12">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" s="26">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L13" s="32"/>
       <c r="O13" s="22">
@@ -2317,47 +2317,47 @@
       </c>
       <c r="C14" s="27">
         <f>C12-C13</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D14" s="12">
         <f t="shared" ref="D14:K14" si="1">D12-INT($D$8/18)-IF(D11&lt;=MOD($D$8,18),1,0)</f>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E14" s="26">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F14" s="27">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G14" s="12">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H14" s="26">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I14" s="27">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J14" s="12">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K14" s="26">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L14" s="34">
         <f>SUM(C14:K14)</f>
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="M14" s="32">
         <f>SUM(C14:K14)-SUM(C$10:K$10)</f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="O14" s="22">
         <v>6</v>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="C15" s="36">
         <f t="shared" ref="C15:K15" si="2">IF(C14&lt;C23,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" s="37">
         <f t="shared" si="2"/>
@@ -2384,11 +2384,11 @@
       </c>
       <c r="E15" s="38">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" s="36">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" s="37">
         <f t="shared" si="2"/>
@@ -2400,15 +2400,15 @@
       </c>
       <c r="I15" s="36">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" s="37">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15" s="38">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" s="12"/>
       <c r="O15" s="22">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="Q15" s="24">
         <f>[1]Schedule!D21</f>
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="2:59" x14ac:dyDescent="0.25">
@@ -2447,7 +2447,7 @@
     </row>
     <row r="17" spans="2:42" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="13" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="C17" s="14" t="s">
         <v>12</v>
@@ -2802,39 +2802,39 @@
         <v>31</v>
       </c>
       <c r="C21" s="29">
+        <v>8</v>
+      </c>
+      <c r="D21" s="30">
         <v>7</v>
       </c>
-      <c r="D21" s="30">
-        <v>10</v>
-      </c>
       <c r="E21" s="31">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F21" s="29">
         <v>8</v>
       </c>
       <c r="G21" s="30">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H21" s="31">
         <v>6</v>
       </c>
       <c r="I21" s="29">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J21" s="30">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K21" s="31">
         <v>7</v>
       </c>
       <c r="L21" s="12">
         <f>SUM(C21:K21)</f>
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="M21" s="32">
         <f>SUM(C21:K21)-SUM(C$10:K$10)</f>
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="O21" s="22">
         <v>13</v>
@@ -2905,15 +2905,15 @@
       </c>
       <c r="C23" s="27">
         <f t="shared" ref="C23:K23" si="4">C21-C22</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D23" s="12">
         <f t="shared" si="4"/>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E23" s="26">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F23" s="27">
         <f t="shared" si="4"/>
@@ -2921,7 +2921,7 @@
       </c>
       <c r="G23" s="12">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H23" s="26">
         <f t="shared" si="4"/>
@@ -2929,11 +2929,11 @@
       </c>
       <c r="I23" s="27">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J23" s="12">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K23" s="26">
         <f t="shared" si="4"/>
@@ -2941,11 +2941,11 @@
       </c>
       <c r="L23" s="34">
         <f>SUM(C23:K23)</f>
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="M23" s="32">
         <f>SUM(C23:K23)-SUM(C$10:K$10)</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="O23" s="22">
         <v>15</v>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="H24" s="38">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" s="36">
         <f t="shared" si="5"/>

</xml_diff>

<commit_message>
Scores: R4 makeup Preston Stoner def. Kaylan Adams 8-0; R5 Kaylan Adams def. Megan Serian 7-1
R4 makeup (4 of 7 recorded): Preston Stoner 8 pts (NET 38) def. Kaylan Adams 0 (NET 50).
R5 (underway): Kaylan Adams 7 pts (NET 48) def. Megan Serian 1 (NET 52).

Standings: Preston Stoner moves to #1 (22.5 pts, 3-1-0). Kaylan Adams up to
12 pts (1-3-1), Megan Serian 11.5 (1-4-0).

apply_overrides: restore Preston Stoner's inherited R1-R3 opponents
(Charlotte Hayes / Jerome Martin / Megan Serian). The score tabs record those
rounds under "Ben Linck", so process_scores can't link them to Preston's
standings entry and nulls his own opponents on every run. New INHERITED_OPPONENTS
override re-applies them, matching prior committed state.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Score Calculator.xlsx
+++ b/Score Calculator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imicompanies-my.sharepoint.com/personal/ehigh_iengtobuild_com/Documents/Documents/Golf League/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="338" documentId="8_{A2D2493B-942A-431B-BFE9-D343A07FD7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36CCB7D5-8C65-423A-825C-6E49503A4E64}"/>
+  <xr:revisionPtr revIDLastSave="370" documentId="8_{A2D2493B-942A-431B-BFE9-D343A07FD7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0CB1F05C-3A2A-41BA-8F4F-14DDBDDD2DF4}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A94AAD03-8B68-4D25-ACDC-485563D823F1}"/>
   </bookViews>
@@ -172,9 +172,6 @@
     <t>Nick Coglianese</t>
   </si>
   <si>
-    <t>Ben Linck</t>
-  </si>
-  <si>
     <t>Charlotte Hayes</t>
   </si>
   <si>
@@ -191,6 +188,9 @@
   </si>
   <si>
     <t>Highland_Creek</t>
+  </si>
+  <si>
+    <t>Preston Stoner</t>
   </si>
 </sst>
 </file>
@@ -581,6 +581,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -604,12 +610,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -664,11 +664,11 @@
       <sheetName val="Oct 14 - 25th"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
       <sheetData sheetId="5">
         <row r="15">
           <cell r="D15">
@@ -712,7 +712,7 @@
         </row>
         <row r="23">
           <cell r="D23">
-            <v>30</v>
+            <v>28</v>
           </cell>
         </row>
         <row r="25">
@@ -741,14 +741,14 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1101,12 +1101,12 @@
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J1" s="39" t="s">
+      <c r="J1" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
     </row>
     <row r="2" spans="2:59" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
@@ -1128,90 +1128,90 @@
         <v>7</v>
       </c>
       <c r="I2" s="5"/>
-      <c r="J2" s="41" t="str">
+      <c r="J2" s="43" t="str">
         <f>B8</f>
-        <v>Charlotte Hayes</v>
-      </c>
-      <c r="K2" s="42"/>
-      <c r="L2" s="43" t="str">
+        <v>Megan Serian</v>
+      </c>
+      <c r="K2" s="44"/>
+      <c r="L2" s="45" t="str">
         <f>B17</f>
-        <v>Megan Serian</v>
-      </c>
-      <c r="M2" s="42"/>
+        <v>Kaylan Adams</v>
+      </c>
+      <c r="M2" s="44"/>
     </row>
     <row r="3" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="44" t="str">
+      <c r="B3" s="46" t="str">
         <f>J2</f>
-        <v>Charlotte Hayes</v>
+        <v>Megan Serian</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="7">
         <f>SUM(C15:E15)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E3" s="7">
         <f>SUM(F15:H15)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F3" s="7">
         <f>SUM(I15:K15)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G3" s="7">
         <f>SUM(C15:K15)</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H3" s="7">
         <f>SUM(C14:K14)</f>
-        <v>41</v>
-      </c>
-      <c r="J3" s="46">
+        <v>52</v>
+      </c>
+      <c r="J3" s="48">
         <f>SUM(D4:H4)</f>
-        <v>8</v>
-      </c>
-      <c r="K3" s="47"/>
-      <c r="L3" s="51">
+        <v>1</v>
+      </c>
+      <c r="K3" s="49"/>
+      <c r="L3" s="53">
         <f>SUM(D6:H6)</f>
-        <v>0</v>
-      </c>
-      <c r="M3" s="47"/>
+        <v>7</v>
+      </c>
+      <c r="M3" s="49"/>
     </row>
     <row r="4" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="45"/>
+      <c r="B4" s="47"/>
       <c r="C4" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="9">
         <f>IF(D3&gt;D5,2,IF(D3=D5,1,0))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" s="9">
         <f>IF(E3&gt;E5,2,IF(E3=E5,1,0))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F4" s="9">
         <f>IF(F3&gt;F5,2,IF(F3=F5,1,0))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G4" s="9">
         <f>IF(G3&gt;G5,1,IF(G3=G5,0.5,0))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" s="9">
         <f>IF(H3&lt;H5,1,IF(H3=H5,0.5,0))</f>
-        <v>1</v>
-      </c>
-      <c r="J4" s="48"/>
-      <c r="K4" s="49"/>
-      <c r="L4" s="52"/>
-      <c r="M4" s="49"/>
+        <v>0</v>
+      </c>
+      <c r="J4" s="50"/>
+      <c r="K4" s="51"/>
+      <c r="L4" s="40"/>
+      <c r="M4" s="51"/>
     </row>
     <row r="5" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="44" t="str">
+      <c r="B5" s="46" t="str">
         <f>L2</f>
-        <v>Megan Serian</v>
+        <v>Kaylan Adams</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>8</v>
@@ -1222,49 +1222,49 @@
       </c>
       <c r="E5" s="11">
         <f>SUM(F24:H24)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="11">
         <f>SUM(I24:K24)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="11">
         <f>SUM(C24:K24)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H5" s="11">
         <f>SUM(C23:K23)</f>
-        <v>54</v>
-      </c>
-      <c r="J5" s="45"/>
-      <c r="K5" s="50"/>
-      <c r="L5" s="40"/>
-      <c r="M5" s="50"/>
+        <v>48</v>
+      </c>
+      <c r="J5" s="47"/>
+      <c r="K5" s="52"/>
+      <c r="L5" s="42"/>
+      <c r="M5" s="52"/>
     </row>
     <row r="6" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="45"/>
+      <c r="B6" s="47"/>
       <c r="C6" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D6" s="9">
         <f>IF(D5&gt;D3,2,IF(D5=D3,1,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="9">
         <f>IF(E5&gt;E3,2,IF(E5=E3,1,0))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F6" s="9">
         <f>IF(F5&gt;F3,2,IF(F5=F3,1,0))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G6" s="9">
         <f>IF(G5&gt;G3,1,IF(G5=G3,0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" s="9">
         <f>IF(H5&lt;H3,1,IF(H5=H3,0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" s="12"/>
       <c r="K6" s="12"/>
@@ -1282,75 +1282,75 @@
       <c r="J7" s="12"/>
       <c r="K7" s="12"/>
       <c r="L7" s="12"/>
-      <c r="T7" s="53" t="s">
-        <v>2</v>
-      </c>
-      <c r="U7" s="52"/>
-      <c r="V7" s="52"/>
-      <c r="W7" s="52"/>
-      <c r="X7" s="52"/>
-      <c r="Y7" s="52"/>
-      <c r="Z7" s="52"/>
-      <c r="AA7" s="52"/>
-      <c r="AB7" s="52"/>
-      <c r="AC7" s="52"/>
-      <c r="AD7" s="52"/>
-      <c r="AE7" s="52"/>
-      <c r="AF7" s="52"/>
-      <c r="AG7" s="52"/>
-      <c r="AH7" s="52"/>
-      <c r="AI7" s="52"/>
-      <c r="AJ7" s="52"/>
-      <c r="AK7" s="52"/>
-      <c r="AL7" s="52"/>
-      <c r="AM7" s="52"/>
-      <c r="AN7" s="53" t="s">
+      <c r="T7" s="39" t="s">
+        <v>2</v>
+      </c>
+      <c r="U7" s="40"/>
+      <c r="V7" s="40"/>
+      <c r="W7" s="40"/>
+      <c r="X7" s="40"/>
+      <c r="Y7" s="40"/>
+      <c r="Z7" s="40"/>
+      <c r="AA7" s="40"/>
+      <c r="AB7" s="40"/>
+      <c r="AC7" s="40"/>
+      <c r="AD7" s="40"/>
+      <c r="AE7" s="40"/>
+      <c r="AF7" s="40"/>
+      <c r="AG7" s="40"/>
+      <c r="AH7" s="40"/>
+      <c r="AI7" s="40"/>
+      <c r="AJ7" s="40"/>
+      <c r="AK7" s="40"/>
+      <c r="AL7" s="40"/>
+      <c r="AM7" s="40"/>
+      <c r="AN7" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="AO7" s="52"/>
-      <c r="AP7" s="52"/>
-      <c r="AQ7" s="52"/>
-      <c r="AR7" s="52"/>
-      <c r="AS7" s="52"/>
-      <c r="AT7" s="52"/>
-      <c r="AU7" s="52"/>
-      <c r="AV7" s="52"/>
-      <c r="AW7" s="52"/>
-      <c r="AX7" s="52"/>
-      <c r="AY7" s="52"/>
-      <c r="AZ7" s="52"/>
-      <c r="BA7" s="52"/>
-      <c r="BB7" s="52"/>
-      <c r="BC7" s="52"/>
-      <c r="BD7" s="52"/>
-      <c r="BE7" s="52"/>
-      <c r="BF7" s="52"/>
-      <c r="BG7" s="52"/>
+      <c r="AO7" s="40"/>
+      <c r="AP7" s="40"/>
+      <c r="AQ7" s="40"/>
+      <c r="AR7" s="40"/>
+      <c r="AS7" s="40"/>
+      <c r="AT7" s="40"/>
+      <c r="AU7" s="40"/>
+      <c r="AV7" s="40"/>
+      <c r="AW7" s="40"/>
+      <c r="AX7" s="40"/>
+      <c r="AY7" s="40"/>
+      <c r="AZ7" s="40"/>
+      <c r="BA7" s="40"/>
+      <c r="BB7" s="40"/>
+      <c r="BC7" s="40"/>
+      <c r="BD7" s="40"/>
+      <c r="BE7" s="40"/>
+      <c r="BF7" s="40"/>
+      <c r="BG7" s="40"/>
     </row>
     <row r="8" spans="2:59" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C8" s="14" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="12">
         <f>_xlfn.XLOOKUP(B8,$P$9:$P$23,$Q$9:$Q$23)</f>
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="12" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="H8" s="12"/>
       <c r="I8" s="12" t="s">
         <v>15</v>
       </c>
       <c r="J8" s="16" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="K8" s="12"/>
       <c r="L8" s="12"/>
@@ -1366,55 +1366,55 @@
       <c r="T8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="U8" s="53" t="s">
+      <c r="U8" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="V8" s="52"/>
-      <c r="W8" s="52"/>
-      <c r="X8" s="52"/>
-      <c r="Y8" s="52"/>
-      <c r="Z8" s="52"/>
-      <c r="AA8" s="52"/>
-      <c r="AB8" s="52"/>
-      <c r="AC8" s="52"/>
-      <c r="AD8" s="53" t="s">
+      <c r="V8" s="40"/>
+      <c r="W8" s="40"/>
+      <c r="X8" s="40"/>
+      <c r="Y8" s="40"/>
+      <c r="Z8" s="40"/>
+      <c r="AA8" s="40"/>
+      <c r="AB8" s="40"/>
+      <c r="AC8" s="40"/>
+      <c r="AD8" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="AE8" s="52"/>
-      <c r="AF8" s="52"/>
-      <c r="AG8" s="52"/>
-      <c r="AH8" s="52"/>
-      <c r="AI8" s="52"/>
-      <c r="AJ8" s="52"/>
-      <c r="AK8" s="52"/>
-      <c r="AL8" s="52"/>
-      <c r="AM8" s="52"/>
+      <c r="AE8" s="40"/>
+      <c r="AF8" s="40"/>
+      <c r="AG8" s="40"/>
+      <c r="AH8" s="40"/>
+      <c r="AI8" s="40"/>
+      <c r="AJ8" s="40"/>
+      <c r="AK8" s="40"/>
+      <c r="AL8" s="40"/>
+      <c r="AM8" s="40"/>
       <c r="AN8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="AO8" s="53" t="s">
+      <c r="AO8" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="AP8" s="52"/>
-      <c r="AQ8" s="52"/>
-      <c r="AR8" s="52"/>
-      <c r="AS8" s="52"/>
-      <c r="AT8" s="52"/>
-      <c r="AU8" s="52"/>
-      <c r="AV8" s="52"/>
-      <c r="AW8" s="52"/>
-      <c r="AX8" s="53" t="s">
+      <c r="AP8" s="40"/>
+      <c r="AQ8" s="40"/>
+      <c r="AR8" s="40"/>
+      <c r="AS8" s="40"/>
+      <c r="AT8" s="40"/>
+      <c r="AU8" s="40"/>
+      <c r="AV8" s="40"/>
+      <c r="AW8" s="40"/>
+      <c r="AX8" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="AY8" s="52"/>
-      <c r="AZ8" s="52"/>
-      <c r="BA8" s="52"/>
-      <c r="BB8" s="52"/>
-      <c r="BC8" s="52"/>
-      <c r="BD8" s="52"/>
-      <c r="BE8" s="52"/>
-      <c r="BF8" s="52"/>
-      <c r="BG8" s="52"/>
+      <c r="AY8" s="40"/>
+      <c r="AZ8" s="40"/>
+      <c r="BA8" s="40"/>
+      <c r="BB8" s="40"/>
+      <c r="BC8" s="40"/>
+      <c r="BD8" s="40"/>
+      <c r="BE8" s="40"/>
+      <c r="BF8" s="40"/>
+      <c r="BG8" s="40"/>
     </row>
     <row r="9" spans="2:59" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="18" t="s">
@@ -1607,7 +1607,7 @@
       $J8="Front 9",INDEX($AO$12:$AW$12,1,D9)
    )
 )</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E10" s="26">
         <f t="array" ref="E10">IF($B$2="Skybrook",
@@ -1620,7 +1620,7 @@
       $J8="Front 9",INDEX($AO$12:$AW$12,1,E9)
    )
 )</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F10" s="27">
         <f t="array" ref="F10">IF($B$2="Skybrook",
@@ -1659,7 +1659,7 @@
       $J8="Front 9",INDEX($AO$12:$AW$12,1,H9)
    )
 )</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I10" s="27">
         <f t="array" ref="I10">IF($B$2="Skybrook",
@@ -1672,7 +1672,7 @@
       $J8="Front 9",INDEX($AO$12:$AW$12,1,I9)
    )
 )</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J10" s="12">
         <f t="array" ref="J10">IF($B$2="Skybrook",
@@ -1685,7 +1685,7 @@
       $J8="Front 9",INDEX($AO$12:$AW$12,1,J9)
    )
 )</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K10" s="26">
         <f t="array" ref="K10">IF($B$2="Skybrook",
@@ -1698,7 +1698,7 @@
       $J8="Front 9",INDEX($AO$12:$AW$12,1,K9)
    )
 )</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L10" s="12">
         <f>SUM(C10:K10)</f>
@@ -1850,7 +1850,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D11" s="12">
         <f t="array" ref="D11">IF($B$2="Skybrook",
@@ -1863,7 +1863,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E11" s="26">
         <f t="array" ref="E11">IF($B$2="Skybrook",
@@ -1876,7 +1876,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="F11" s="27">
         <f t="array" ref="F11">IF($B$2="Skybrook",
@@ -1889,7 +1889,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G11" s="12">
         <f t="array" ref="G11">IF($B$2="Skybrook",
@@ -1902,7 +1902,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H11" s="26">
         <f t="array" ref="H11">IF($B$2="Skybrook",
@@ -1915,7 +1915,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I11" s="27">
         <f t="array" ref="I11">IF($B$2="Skybrook",
@@ -1928,7 +1928,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J11" s="12">
         <f t="array" ref="J11">IF($B$2="Skybrook",
@@ -1941,7 +1941,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K11" s="26">
         <f t="array" ref="K11">IF($B$2="Skybrook",
@@ -1954,7 +1954,7 @@
       $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="L11" s="12"/>
       <c r="O11" s="22">
@@ -2094,22 +2094,22 @@
         <v>31</v>
       </c>
       <c r="C12" s="29">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D12" s="30">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E12" s="31">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F12" s="29">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G12" s="30">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H12" s="31">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I12" s="29">
         <v>8</v>
@@ -2118,15 +2118,15 @@
         <v>6</v>
       </c>
       <c r="K12" s="31">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L12" s="12">
         <f>SUM(C12:K12)</f>
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="M12" s="32">
         <f>SUM(C12:K12)-SUM(C$10:K$10)</f>
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="O12" s="22">
         <v>4</v>
@@ -2265,15 +2265,15 @@
       </c>
       <c r="C13" s="27">
         <f t="shared" ref="C13:K13" si="0">INT($D$8/18)+IF(C11&lt;=MOD($D$8,18),1,0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" s="12">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" s="26">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="27">
         <f t="shared" si="0"/>
@@ -2281,23 +2281,23 @@
       </c>
       <c r="G13" s="12">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H13" s="26">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I13" s="27">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J13" s="12">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="26">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L13" s="32"/>
       <c r="O13" s="22">
@@ -2317,47 +2317,47 @@
       </c>
       <c r="C14" s="27">
         <f>C12-C13</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D14" s="12">
         <f t="shared" ref="D14:K14" si="1">D12-INT($D$8/18)-IF(D11&lt;=MOD($D$8,18),1,0)</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E14" s="26">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F14" s="27">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G14" s="12">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H14" s="26">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I14" s="27">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J14" s="12">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K14" s="26">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L14" s="34">
         <f>SUM(C14:K14)</f>
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="M14" s="32">
         <f>SUM(C14:K14)-SUM(C$10:K$10)</f>
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="O14" s="22">
         <v>6</v>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="C15" s="36">
         <f t="shared" ref="C15:K15" si="2">IF(C14&lt;C23,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" s="37">
         <f t="shared" si="2"/>
@@ -2384,31 +2384,31 @@
       </c>
       <c r="E15" s="38">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" s="36">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" s="37">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H15" s="38">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15" s="36">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" s="37">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" s="38">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15" s="12"/>
       <c r="O15" s="22">
@@ -2447,7 +2447,7 @@
     </row>
     <row r="17" spans="2:42" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="13" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C17" s="14" t="s">
         <v>12</v>
@@ -2461,7 +2461,7 @@
         <v>13</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="H17" s="12"/>
       <c r="I17" s="12" t="s">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="J17" s="12" t="str">
         <f>J8</f>
-        <v>Front 9</v>
+        <v>Back 9</v>
       </c>
       <c r="K17" s="12"/>
       <c r="L17" s="12"/>
@@ -2477,11 +2477,11 @@
         <v>9</v>
       </c>
       <c r="P17" s="23" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="Q17" s="24">
         <f>[1]Schedule!D23</f>
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="2:42" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="P18" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q18" s="24">
         <v>20</v>
@@ -2555,7 +2555,7 @@
       $J17="Front 9",INDEX($AO$12:$AW$12,1,D18)
    )
 )</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E19" s="26">
         <f t="array" ref="E19">IF($B$2="Skybrook",
@@ -2568,7 +2568,7 @@
       $J17="Front 9",INDEX($AO$12:$AW$12,1,E18)
    )
 )</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F19" s="27">
         <f t="array" ref="F19">IF($B$2="Skybrook",
@@ -2607,7 +2607,7 @@
       $J17="Front 9",INDEX($AO$12:$AW$12,1,H18)
    )
 )</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I19" s="27">
         <f t="array" ref="I19">IF($B$2="Skybrook",
@@ -2620,7 +2620,7 @@
       $J17="Front 9",INDEX($AO$12:$AW$12,1,I18)
    )
 )</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J19" s="12">
         <f t="array" ref="J19">IF($B$2="Skybrook",
@@ -2633,7 +2633,7 @@
       $J17="Front 9",INDEX($AO$12:$AW$12,1,J18)
    )
 )</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K19" s="26">
         <f t="array" ref="K19">IF($B$2="Skybrook",
@@ -2646,7 +2646,7 @@
       $J17="Front 9",INDEX($AO$12:$AW$12,1,K18)
    )
 )</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L19" s="12">
         <f>SUM(C19:K19)</f>
@@ -2657,7 +2657,7 @@
         <v>11</v>
       </c>
       <c r="P19" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q19" s="24">
         <f>[1]Schedule!D25</f>
@@ -2679,7 +2679,7 @@
       $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D20" s="12">
         <f t="array" ref="D20">IF($B$2="Skybrook",
@@ -2692,7 +2692,7 @@
       $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E20" s="26">
         <f t="array" ref="E20">IF($B$2="Skybrook",
@@ -2705,7 +2705,7 @@
       $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="F20" s="27">
         <f t="array" ref="F20">IF($B$2="Skybrook",
@@ -2718,7 +2718,7 @@
       $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G20" s="12">
         <f t="array" ref="G20">IF($B$2="Skybrook",
@@ -2731,7 +2731,7 @@
       $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H20" s="26">
         <f t="array" ref="H20">IF($B$2="Skybrook",
@@ -2744,7 +2744,7 @@
       $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I20" s="27">
         <f t="array" ref="I20">IF($B$2="Skybrook",
@@ -2757,7 +2757,7 @@
       $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J20" s="12">
         <f t="array" ref="J20">IF($B$2="Skybrook",
@@ -2770,7 +2770,7 @@
       $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K20" s="26">
         <f t="array" ref="K20">IF($B$2="Skybrook",
@@ -2783,14 +2783,14 @@
       $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
    )
 )</f>
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="L20" s="12"/>
       <c r="O20" s="22">
         <v>12</v>
       </c>
       <c r="P20" s="23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q20" s="24">
         <f>[1]Schedule!D26</f>
@@ -2805,42 +2805,42 @@
         <v>8</v>
       </c>
       <c r="D21" s="30">
+        <v>6</v>
+      </c>
+      <c r="E21" s="31">
         <v>10</v>
-      </c>
-      <c r="E21" s="31">
-        <v>6</v>
       </c>
       <c r="F21" s="29">
         <v>8</v>
       </c>
       <c r="G21" s="30">
+        <v>5</v>
+      </c>
+      <c r="H21" s="31">
         <v>8</v>
       </c>
-      <c r="H21" s="31">
+      <c r="I21" s="29">
+        <v>8</v>
+      </c>
+      <c r="J21" s="30">
         <v>6</v>
       </c>
-      <c r="I21" s="29">
-        <v>10</v>
-      </c>
-      <c r="J21" s="30">
-        <v>8</v>
-      </c>
       <c r="K21" s="31">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L21" s="12">
         <f>SUM(C21:K21)</f>
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="M21" s="32">
         <f>SUM(C21:K21)-SUM(C$10:K$10)</f>
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="O21" s="22">
         <v>13</v>
       </c>
       <c r="P21" s="23" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Q21" s="24">
         <f>[1]Schedule!D27</f>
@@ -2892,7 +2892,7 @@
         <v>14</v>
       </c>
       <c r="P22" s="23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="Q22" s="24">
         <f>[1]Schedule!D28</f>
@@ -2909,11 +2909,11 @@
       </c>
       <c r="D23" s="12">
         <f t="shared" si="4"/>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E23" s="26">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F23" s="27">
         <f t="shared" si="4"/>
@@ -2921,31 +2921,31 @@
       </c>
       <c r="G23" s="12">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H23" s="26">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I23" s="27">
         <f t="shared" si="4"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J23" s="12">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K23" s="26">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L23" s="34">
         <f>SUM(C23:K23)</f>
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="M23" s="32">
         <f>SUM(C23:K23)-SUM(C$10:K$10)</f>
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="O23" s="22">
         <v>15</v>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="G24" s="37">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H24" s="38">
         <f t="shared" si="5"/>
@@ -2996,7 +2996,7 @@
       </c>
       <c r="K24" s="38">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" s="12"/>
     </row>
@@ -3007,12 +3007,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="T7:AM7"/>
-    <mergeCell ref="AN7:BG7"/>
-    <mergeCell ref="U8:AC8"/>
-    <mergeCell ref="AD8:AM8"/>
-    <mergeCell ref="AO8:AW8"/>
-    <mergeCell ref="AX8:BG8"/>
     <mergeCell ref="J1:M1"/>
     <mergeCell ref="J2:K2"/>
     <mergeCell ref="L2:M2"/>
@@ -3020,6 +3014,12 @@
     <mergeCell ref="J3:K5"/>
     <mergeCell ref="L3:M5"/>
     <mergeCell ref="B5:B6"/>
+    <mergeCell ref="T7:AM7"/>
+    <mergeCell ref="AN7:BG7"/>
+    <mergeCell ref="U8:AC8"/>
+    <mergeCell ref="AD8:AM8"/>
+    <mergeCell ref="AO8:AW8"/>
+    <mergeCell ref="AX8:BG8"/>
   </mergeCells>
   <conditionalFormatting sqref="C15:K15 C24:K24">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
@@ -3058,7 +3058,7 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="3:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Scores: R3 Ethan High def. Michael McHugh 7-1 (Warrior GC); R5 Jerome Martin def. Nick Coglianese 6-2
- R3 makeup @ Warrior Golf Club: Ethan High 7 pts (NET 35) def. Michael McHugh 1 pt (NET 43)
- R5 @ Skybrook: Jerome Martin 6 pts (NET 52) def. Nick Coglianese 2 pts (NET 54)
- Standings re-sorted: Ethan High to #1 (27 pts, 4-0-0); Jerome edges Alex for #7 on fewer losses
- Score Calculator: wired Warrior Golf Club into PAR/HC course lookups (2-way -> 3-way IFS) + added Warrior_Golf_Club named range and Helper tee list

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Score Calculator.xlsx
+++ b/Score Calculator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imicompanies-my.sharepoint.com/personal/ehigh_iengtobuild_com/Documents/Documents/Golf League/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="370" documentId="8_{A2D2493B-942A-431B-BFE9-D343A07FD7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0CB1F05C-3A2A-41BA-8F4F-14DDBDDD2DF4}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="11_D812028DA688F3B9538958C5B423B5CF7585794A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C91DDDA-963D-45B0-B6C6-5451DA767290}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A94AAD03-8B68-4D25-ACDC-485563D823F1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculator" sheetId="1" r:id="rId1"/>
@@ -22,12 +22,11 @@
   <definedNames>
     <definedName name="Highland_Creek">Helper!$D$3:$D$5</definedName>
     <definedName name="Skybrook">Helper!$C$3:$C$5</definedName>
+    <definedName name="Warrior_Golf_Club">Helper!$E$3:$E$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -39,15 +38,12 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="51">
   <si>
     <t>Fill in the course, your name, tees, front/back and gross scores in the grey boxes</t>
   </si>
@@ -55,121 +51,133 @@
     <t>Points</t>
   </si>
   <si>
+    <t>Warrior Golf Club</t>
+  </si>
+  <si>
+    <t>First 3</t>
+  </si>
+  <si>
+    <t>Middle 3</t>
+  </si>
+  <si>
+    <t>Final 3</t>
+  </si>
+  <si>
+    <t>Overall</t>
+  </si>
+  <si>
+    <t>Net Score</t>
+  </si>
+  <si>
+    <t>Holes Won</t>
+  </si>
+  <si>
+    <t>PTS</t>
+  </si>
+  <si>
     <t>Skybrook</t>
   </si>
   <si>
-    <t>First 3</t>
-  </si>
-  <si>
-    <t>Middle 3</t>
-  </si>
-  <si>
-    <t>Final 3</t>
-  </si>
-  <si>
-    <t>Overall</t>
-  </si>
-  <si>
-    <t>Net Score</t>
-  </si>
-  <si>
-    <t>Holes Won</t>
-  </si>
-  <si>
-    <t>PTS</t>
-  </si>
-  <si>
     <t>Highland Creek</t>
   </si>
   <si>
+    <t>Nick Coglianese</t>
+  </si>
+  <si>
+    <t>Handicap:</t>
+  </si>
+  <si>
+    <t>Tees:</t>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>Holes:</t>
+  </si>
+  <si>
+    <t>Front 9</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Handicap</t>
+  </si>
+  <si>
+    <t>HC's by Tees</t>
+  </si>
+  <si>
+    <t>Back 9</t>
+  </si>
+  <si>
+    <t>HOLE</t>
+  </si>
+  <si>
+    <t>Brian Wojcio</t>
+  </si>
+  <si>
+    <t>Black</t>
+  </si>
+  <si>
+    <t>PAR</t>
+  </si>
+  <si>
+    <t>Ethan High</t>
+  </si>
+  <si>
+    <t>Green</t>
+  </si>
+  <si>
+    <t>White</t>
+  </si>
+  <si>
+    <t>HC</t>
+  </si>
+  <si>
+    <t>Rob Bass</t>
+  </si>
+  <si>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>GROSS</t>
+  </si>
+  <si>
+    <t>Carson Bass</t>
+  </si>
+  <si>
+    <t>Par</t>
+  </si>
+  <si>
+    <t>Strokes</t>
+  </si>
+  <si>
+    <t>Michael McHugh</t>
+  </si>
+  <si>
+    <t>NET</t>
+  </si>
+  <si>
+    <t>Bruce Atkins</t>
+  </si>
+  <si>
+    <t>Wins Hole</t>
+  </si>
+  <si>
+    <t>Alex Palmer</t>
+  </si>
+  <si>
     <t>Curtis Lynn</t>
   </si>
   <si>
-    <t>Handicap:</t>
-  </si>
-  <si>
-    <t>Tees:</t>
-  </si>
-  <si>
-    <t>Blue</t>
-  </si>
-  <si>
-    <t>Holes:</t>
-  </si>
-  <si>
-    <t>Front 9</t>
-  </si>
-  <si>
-    <t>#</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Handicap</t>
-  </si>
-  <si>
-    <t>HC's by Tees</t>
-  </si>
-  <si>
-    <t>Back 9</t>
-  </si>
-  <si>
-    <t>HOLE</t>
-  </si>
-  <si>
-    <t>Brian Wojcio</t>
-  </si>
-  <si>
-    <t>PAR</t>
-  </si>
-  <si>
-    <t>Ethan High</t>
-  </si>
-  <si>
-    <t>Green</t>
-  </si>
-  <si>
-    <t>White</t>
-  </si>
-  <si>
-    <t>HC</t>
-  </si>
-  <si>
-    <t>Rob Bass</t>
-  </si>
-  <si>
-    <t>Red</t>
-  </si>
-  <si>
-    <t>GROSS</t>
-  </si>
-  <si>
-    <t>Carson Bass</t>
-  </si>
-  <si>
-    <t>Par</t>
-  </si>
-  <si>
-    <t>Strokes</t>
-  </si>
-  <si>
-    <t>Michael McHugh</t>
-  </si>
-  <si>
-    <t>NET</t>
-  </si>
-  <si>
-    <t>Bruce Atkins</t>
-  </si>
-  <si>
-    <t>Wins Hole</t>
-  </si>
-  <si>
-    <t>Alex Palmer</t>
-  </si>
-  <si>
-    <t>Nick Coglianese</t>
+    <t>Jerome Martin</t>
+  </si>
+  <si>
+    <t>Preston Stoner</t>
   </si>
   <si>
     <t>Charlotte Hayes</t>
@@ -178,9 +186,6 @@
     <t>David Maddox</t>
   </si>
   <si>
-    <t>Jerome Martin</t>
-  </si>
-  <si>
     <t>Kaylan Adams</t>
   </si>
   <si>
@@ -190,7 +195,7 @@
     <t>Highland_Creek</t>
   </si>
   <si>
-    <t>Preston Stoner</t>
+    <t>Warrior_Golf_Club</t>
   </si>
 </sst>
 </file>
@@ -587,35 +592,35 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 3 2" xfId="1" xr:uid="{64D002C7-EAB9-4170-909D-6BC7434A7F9C}"/>
+    <cellStyle name="Normal 3 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -644,9 +649,6 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Scores 2024"/>
       <sheetName val="Sep 2 - 13th"/>
@@ -664,11 +666,11 @@
       <sheetName val="Oct 14 - 25th"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
       <sheetData sheetId="5">
         <row r="15">
           <cell r="D15">
@@ -741,14 +743,14 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1070,8 +1072,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C7E9C1E-B4F8-42BE-ADD6-CFDCDE6729D4}">
-  <dimension ref="B1:BG29"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B1:CA24"/>
   <sheetFormatPr defaultColWidth="9.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.5703125" style="2" customWidth="1"/>
@@ -1093,24 +1095,28 @@
     <col min="41" max="49" width="4" style="2" customWidth="1"/>
     <col min="50" max="50" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="51" max="59" width="4" style="2" customWidth="1"/>
-    <col min="60" max="65" width="9.85546875" style="2" customWidth="1"/>
-    <col min="66" max="16384" width="9.85546875" style="2"/>
+    <col min="60" max="60" width="11" style="2" bestFit="1" customWidth="1"/>
+    <col min="61" max="69" width="4" style="2" customWidth="1"/>
+    <col min="70" max="70" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="71" max="79" width="4" style="2" customWidth="1"/>
+    <col min="80" max="80" width="9.85546875" style="2" customWidth="1"/>
+    <col min="81" max="16384" width="9.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:79" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J1" s="41" t="s">
-        <v>1</v>
-      </c>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
+      <c r="J1" s="51" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="52"/>
+      <c r="L1" s="52"/>
+      <c r="M1" s="52"/>
     </row>
-    <row r="2" spans="2:59" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:79" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>3</v>
@@ -1128,90 +1134,90 @@
         <v>7</v>
       </c>
       <c r="I2" s="5"/>
-      <c r="J2" s="43" t="str">
+      <c r="J2" s="49" t="str">
         <f>B8</f>
-        <v>Megan Serian</v>
-      </c>
-      <c r="K2" s="44"/>
-      <c r="L2" s="45" t="str">
+        <v>Ethan High</v>
+      </c>
+      <c r="K2" s="42"/>
+      <c r="L2" s="41" t="str">
         <f>B17</f>
-        <v>Kaylan Adams</v>
-      </c>
-      <c r="M2" s="44"/>
+        <v>Michael McHugh</v>
+      </c>
+      <c r="M2" s="42"/>
     </row>
-    <row r="3" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="46" t="str">
+    <row r="3" spans="2:79" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="50" t="str">
         <f>J2</f>
-        <v>Megan Serian</v>
+        <v>Ethan High</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="7">
         <f>SUM(C15:E15)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E3" s="7">
         <f>SUM(F15:H15)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F3" s="7">
         <f>SUM(I15:K15)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="7">
         <f>SUM(C15:K15)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H3" s="7">
         <f>SUM(C14:K14)</f>
-        <v>52</v>
-      </c>
-      <c r="J3" s="48">
+        <v>35</v>
+      </c>
+      <c r="J3" s="43">
         <f>SUM(D4:H4)</f>
-        <v>1</v>
-      </c>
-      <c r="K3" s="49"/>
+        <v>7</v>
+      </c>
+      <c r="K3" s="44"/>
       <c r="L3" s="53">
         <f>SUM(D6:H6)</f>
-        <v>7</v>
-      </c>
-      <c r="M3" s="49"/>
+        <v>1</v>
+      </c>
+      <c r="M3" s="44"/>
     </row>
-    <row r="4" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:79" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B4" s="47"/>
       <c r="C4" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="9">
         <f>IF(D3&gt;D5,2,IF(D3=D5,1,0))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="9">
         <f>IF(E3&gt;E5,2,IF(E3=E5,1,0))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F4" s="9">
         <f>IF(F3&gt;F5,2,IF(F3=F5,1,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" s="9">
         <f>IF(G3&gt;G5,1,IF(G3=G5,0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="9">
         <f>IF(H3&lt;H5,1,IF(H3=H5,0.5,0))</f>
-        <v>0</v>
-      </c>
-      <c r="J4" s="50"/>
-      <c r="K4" s="51"/>
+        <v>1</v>
+      </c>
+      <c r="J4" s="45"/>
+      <c r="K4" s="46"/>
       <c r="L4" s="40"/>
-      <c r="M4" s="51"/>
+      <c r="M4" s="46"/>
     </row>
-    <row r="5" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="46" t="str">
+    <row r="5" spans="2:79" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="50" t="str">
         <f>L2</f>
-        <v>Kaylan Adams</v>
+        <v>Michael McHugh</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>8</v>
@@ -1234,44 +1240,44 @@
       </c>
       <c r="H5" s="11">
         <f>SUM(C23:K23)</f>
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="J5" s="47"/>
-      <c r="K5" s="52"/>
-      <c r="L5" s="42"/>
-      <c r="M5" s="52"/>
+      <c r="K5" s="48"/>
+      <c r="L5" s="52"/>
+      <c r="M5" s="48"/>
     </row>
-    <row r="6" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:79" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B6" s="47"/>
       <c r="C6" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D6" s="9">
         <f>IF(D5&gt;D3,2,IF(D5=D3,1,0))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="9">
         <f>IF(E5&gt;E3,2,IF(E5=E3,1,0))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F6" s="9">
         <f>IF(F5&gt;F3,2,IF(F5=F3,1,0))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" s="9">
         <f>IF(G5&gt;G3,1,IF(G5=G3,0.5,0))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" s="9">
         <f>IF(H5&lt;H3,1,IF(H5=H3,0.5,0))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" s="12"/>
       <c r="K6" s="12"/>
       <c r="L6" s="12"/>
       <c r="M6" s="12"/>
     </row>
-    <row r="7" spans="2:59" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:79" x14ac:dyDescent="0.2">
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
       <c r="E7" s="12"/>
@@ -1283,7 +1289,7 @@
       <c r="K7" s="12"/>
       <c r="L7" s="12"/>
       <c r="T7" s="39" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="U7" s="40"/>
       <c r="V7" s="40"/>
@@ -1305,7 +1311,7 @@
       <c r="AL7" s="40"/>
       <c r="AM7" s="40"/>
       <c r="AN7" s="39" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AO7" s="40"/>
       <c r="AP7" s="40"/>
@@ -1326,48 +1332,70 @@
       <c r="BE7" s="40"/>
       <c r="BF7" s="40"/>
       <c r="BG7" s="40"/>
+      <c r="BH7" s="39" t="s">
+        <v>2</v>
+      </c>
+      <c r="BI7" s="40"/>
+      <c r="BJ7" s="40"/>
+      <c r="BK7" s="40"/>
+      <c r="BL7" s="40"/>
+      <c r="BM7" s="40"/>
+      <c r="BN7" s="40"/>
+      <c r="BO7" s="40"/>
+      <c r="BP7" s="40"/>
+      <c r="BQ7" s="40"/>
+      <c r="BR7" s="40"/>
+      <c r="BS7" s="40"/>
+      <c r="BT7" s="40"/>
+      <c r="BU7" s="40"/>
+      <c r="BV7" s="40"/>
+      <c r="BW7" s="40"/>
+      <c r="BX7" s="40"/>
+      <c r="BY7" s="40"/>
+      <c r="BZ7" s="40"/>
+      <c r="CA7" s="40"/>
     </row>
-    <row r="8" spans="2:59" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:79" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="13" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D8" s="12">
         <f>_xlfn.XLOOKUP(B8,$P$9:$P$23,$Q$9:$Q$23)</f>
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H8" s="12"/>
       <c r="I8" s="12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J8" s="16" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="K8" s="12"/>
       <c r="L8" s="12"/>
       <c r="O8" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="P8" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q8" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="T8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="U8" s="39" t="s">
         <v>17</v>
-      </c>
-      <c r="P8" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q8" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="T8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="U8" s="39" t="s">
-        <v>16</v>
       </c>
       <c r="V8" s="40"/>
       <c r="W8" s="40"/>
@@ -1378,7 +1406,7 @@
       <c r="AB8" s="40"/>
       <c r="AC8" s="40"/>
       <c r="AD8" s="39" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="AE8" s="40"/>
       <c r="AF8" s="40"/>
@@ -1390,10 +1418,10 @@
       <c r="AL8" s="40"/>
       <c r="AM8" s="40"/>
       <c r="AN8" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="AO8" s="39" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AP8" s="40"/>
       <c r="AQ8" s="40"/>
@@ -1404,7 +1432,7 @@
       <c r="AV8" s="40"/>
       <c r="AW8" s="40"/>
       <c r="AX8" s="39" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="AY8" s="40"/>
       <c r="AZ8" s="40"/>
@@ -1415,10 +1443,36 @@
       <c r="BE8" s="40"/>
       <c r="BF8" s="40"/>
       <c r="BG8" s="40"/>
+      <c r="BH8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="BI8" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="BJ8" s="40"/>
+      <c r="BK8" s="40"/>
+      <c r="BL8" s="40"/>
+      <c r="BM8" s="40"/>
+      <c r="BN8" s="40"/>
+      <c r="BO8" s="40"/>
+      <c r="BP8" s="40"/>
+      <c r="BQ8" s="40"/>
+      <c r="BR8" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="BS8" s="40"/>
+      <c r="BT8" s="40"/>
+      <c r="BU8" s="40"/>
+      <c r="BV8" s="40"/>
+      <c r="BW8" s="40"/>
+      <c r="BX8" s="40"/>
+      <c r="BY8" s="40"/>
+      <c r="BZ8" s="40"/>
+      <c r="CA8" s="40"/>
     </row>
-    <row r="9" spans="2:59" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:79" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="18" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C9" s="19">
         <v>1</v>
@@ -1452,14 +1506,14 @@
         <v>1</v>
       </c>
       <c r="P9" s="23" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q9" s="24">
         <f>[1]Schedule!D15</f>
         <v>12</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="U9" s="12">
         <v>7</v>
@@ -1489,7 +1543,7 @@
         <v>1</v>
       </c>
       <c r="AD9" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AE9" s="12">
         <v>4</v>
@@ -1519,7 +1573,7 @@
         <v>10</v>
       </c>
       <c r="AN9" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AO9" s="12">
         <v>7</v>
@@ -1549,7 +1603,7 @@
         <v>3</v>
       </c>
       <c r="AX9" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AY9" s="12">
         <v>14</v>
@@ -1578,144 +1632,123 @@
       <c r="BG9" s="12">
         <v>18</v>
       </c>
+      <c r="BH9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="BI9" s="12">
+        <v>7</v>
+      </c>
+      <c r="BJ9" s="12">
+        <v>3</v>
+      </c>
+      <c r="BK9" s="12">
+        <v>13</v>
+      </c>
+      <c r="BL9" s="12">
+        <v>9</v>
+      </c>
+      <c r="BM9" s="12">
+        <v>11</v>
+      </c>
+      <c r="BN9" s="12">
+        <v>15</v>
+      </c>
+      <c r="BO9" s="12">
+        <v>1</v>
+      </c>
+      <c r="BP9" s="12">
+        <v>5</v>
+      </c>
+      <c r="BQ9" s="12">
+        <v>17</v>
+      </c>
+      <c r="BR9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="BS9" s="12">
+        <v>2</v>
+      </c>
+      <c r="BT9" s="12">
+        <v>6</v>
+      </c>
+      <c r="BU9" s="12">
+        <v>12</v>
+      </c>
+      <c r="BV9" s="12">
+        <v>14</v>
+      </c>
+      <c r="BW9" s="12">
+        <v>16</v>
+      </c>
+      <c r="BX9" s="12">
+        <v>18</v>
+      </c>
+      <c r="BY9" s="12">
+        <v>8</v>
+      </c>
+      <c r="BZ9" s="12">
+        <v>4</v>
+      </c>
+      <c r="CA9" s="12">
+        <v>10</v>
+      </c>
     </row>
-    <row r="10" spans="2:59" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:79" x14ac:dyDescent="0.25">
       <c r="B10" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C10" s="12">
-        <f t="array" ref="C10">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AE$12:$AM$12,1,C9),
-      $J8="Front 9",INDEX($U$12:$AC$12,1,C9)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AY$12:$BG$12,1,C9),
-      $J8="Front 9",INDEX($AO$12:$AW$12,1,C9)
-   )
-)</f>
-        <v>4</v>
+        <f t="array" ref="C10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,C9),$J8="Front 9",INDEX($U$12:$AC$12,1,C9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,C9),$J8="Front 9",INDEX($AO$12:$AW$12,1,C9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,C9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,C9)))</f>
+        <v>5</v>
       </c>
       <c r="D10" s="12">
-        <f t="array" ref="D10">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AE$12:$AM$12,1,D9),
-      $J8="Front 9",INDEX($U$12:$AC$12,1,D9)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AY$12:$BG$12,1,D9),
-      $J8="Front 9",INDEX($AO$12:$AW$12,1,D9)
-   )
-)</f>
-        <v>3</v>
+        <f t="array" ref="D10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,D9),$J8="Front 9",INDEX($U$12:$AC$12,1,D9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,D9),$J8="Front 9",INDEX($AO$12:$AW$12,1,D9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,D9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,D9)))</f>
+        <v>4</v>
       </c>
       <c r="E10" s="26">
-        <f t="array" ref="E10">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AE$12:$AM$12,1,E9),
-      $J8="Front 9",INDEX($U$12:$AC$12,1,E9)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AY$12:$BG$12,1,E9),
-      $J8="Front 9",INDEX($AO$12:$AW$12,1,E9)
-   )
-)</f>
-        <v>5</v>
+        <f t="array" ref="E10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,E9),$J8="Front 9",INDEX($U$12:$AC$12,1,E9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,E9),$J8="Front 9",INDEX($AO$12:$AW$12,1,E9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,E9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,E9)))</f>
+        <v>3</v>
       </c>
       <c r="F10" s="27">
-        <f t="array" ref="F10">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AE$12:$AM$12,1,F9),
-      $J8="Front 9",INDEX($U$12:$AC$12,1,F9)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AY$12:$BG$12,1,F9),
-      $J8="Front 9",INDEX($AO$12:$AW$12,1,F9)
-   )
-)</f>
-        <v>4</v>
+        <f t="array" ref="F10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,F9),$J8="Front 9",INDEX($U$12:$AC$12,1,F9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,F9),$J8="Front 9",INDEX($AO$12:$AW$12,1,F9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,F9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,F9)))</f>
+        <v>5</v>
       </c>
       <c r="G10" s="12">
-        <f t="array" ref="G10">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AE$12:$AM$12,1,G9),
-      $J8="Front 9",INDEX($U$12:$AC$12,1,G9)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AY$12:$BG$12,1,G9),
-      $J8="Front 9",INDEX($AO$12:$AW$12,1,G9)
-   )
-)</f>
+        <f t="array" ref="G10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,G9),$J8="Front 9",INDEX($U$12:$AC$12,1,G9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,G9),$J8="Front 9",INDEX($AO$12:$AW$12,1,G9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,G9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,G9)))</f>
         <v>4</v>
       </c>
       <c r="H10" s="26">
-        <f t="array" ref="H10">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AE$12:$AM$12,1,H9),
-      $J8="Front 9",INDEX($U$12:$AC$12,1,H9)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AY$12:$BG$12,1,H9),
-      $J8="Front 9",INDEX($AO$12:$AW$12,1,H9)
-   )
-)</f>
-        <v>4</v>
+        <f t="array" ref="H10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,H9),$J8="Front 9",INDEX($U$12:$AC$12,1,H9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,H9),$J8="Front 9",INDEX($AO$12:$AW$12,1,H9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,H9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,H9)))</f>
+        <v>3</v>
       </c>
       <c r="I10" s="27">
-        <f t="array" ref="I10">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AE$12:$AM$12,1,I9),
-      $J8="Front 9",INDEX($U$12:$AC$12,1,I9)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AY$12:$BG$12,1,I9),
-      $J8="Front 9",INDEX($AO$12:$AW$12,1,I9)
-   )
-)</f>
+        <f t="array" ref="I10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,I9),$J8="Front 9",INDEX($U$12:$AC$12,1,I9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,I9),$J8="Front 9",INDEX($AO$12:$AW$12,1,I9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,I9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,I9)))</f>
         <v>4</v>
       </c>
       <c r="J10" s="12">
-        <f t="array" ref="J10">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AE$12:$AM$12,1,J9),
-      $J8="Front 9",INDEX($U$12:$AC$12,1,J9)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AY$12:$BG$12,1,J9),
-      $J8="Front 9",INDEX($AO$12:$AW$12,1,J9)
-   )
-)</f>
+        <f t="array" ref="J10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,J9),$J8="Front 9",INDEX($U$12:$AC$12,1,J9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,J9),$J8="Front 9",INDEX($AO$12:$AW$12,1,J9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,J9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,J9)))</f>
         <v>3</v>
       </c>
       <c r="K10" s="26">
-        <f t="array" ref="K10">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AE$12:$AM$12,1,K9),
-      $J8="Front 9",INDEX($U$12:$AC$12,1,K9)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",INDEX($AY$12:$BG$12,1,K9),
-      $J8="Front 9",INDEX($AO$12:$AW$12,1,K9)
-   )
-)</f>
-        <v>5</v>
+        <f t="array" ref="K10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,K9),$J8="Front 9",INDEX($U$12:$AC$12,1,K9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,K9),$J8="Front 9",INDEX($AO$12:$AW$12,1,K9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,K9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,K9)))</f>
+        <v>4</v>
       </c>
       <c r="L10" s="12">
         <f>SUM(C10:K10)</f>
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O10" s="22">
         <v>2</v>
       </c>
       <c r="P10" s="23" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="Q10" s="24">
         <f>[1]Schedule!D16</f>
         <v>12</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="U10" s="12">
         <v>7</v>
@@ -1745,7 +1778,7 @@
         <v>1</v>
       </c>
       <c r="AD10" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="AE10" s="12">
         <v>4</v>
@@ -1775,7 +1808,7 @@
         <v>10</v>
       </c>
       <c r="AN10" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="AO10" s="12">
         <v>7</v>
@@ -1805,7 +1838,7 @@
         <v>3</v>
       </c>
       <c r="AX10" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="AY10" s="12">
         <v>14</v>
@@ -1834,127 +1867,106 @@
       <c r="BG10" s="12">
         <v>18</v>
       </c>
+      <c r="BH10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="BI10" s="12">
+        <v>7</v>
+      </c>
+      <c r="BJ10" s="12">
+        <v>3</v>
+      </c>
+      <c r="BK10" s="12">
+        <v>13</v>
+      </c>
+      <c r="BL10" s="12">
+        <v>9</v>
+      </c>
+      <c r="BM10" s="12">
+        <v>11</v>
+      </c>
+      <c r="BN10" s="12">
+        <v>15</v>
+      </c>
+      <c r="BO10" s="12">
+        <v>1</v>
+      </c>
+      <c r="BP10" s="12">
+        <v>5</v>
+      </c>
+      <c r="BQ10" s="12">
+        <v>17</v>
+      </c>
+      <c r="BR10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="BS10" s="12">
+        <v>2</v>
+      </c>
+      <c r="BT10" s="12">
+        <v>6</v>
+      </c>
+      <c r="BU10" s="12">
+        <v>12</v>
+      </c>
+      <c r="BV10" s="12">
+        <v>14</v>
+      </c>
+      <c r="BW10" s="12">
+        <v>16</v>
+      </c>
+      <c r="BX10" s="12">
+        <v>18</v>
+      </c>
+      <c r="BY10" s="12">
+        <v>8</v>
+      </c>
+      <c r="BZ10" s="12">
+        <v>4</v>
+      </c>
+      <c r="CA10" s="12">
+        <v>10</v>
+      </c>
     </row>
-    <row r="11" spans="2:59" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:79" x14ac:dyDescent="0.25">
       <c r="B11" s="25" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C11" s="12">
-        <f t="array" ref="C11">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>14</v>
+        <f t="array" ref="C11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>7</v>
       </c>
       <c r="D11" s="12">
-        <f t="array" ref="D11">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>8</v>
+        <f t="array" ref="D11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>3</v>
       </c>
       <c r="E11" s="26">
-        <f t="array" ref="E11">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>6</v>
+        <f t="array" ref="E11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>13</v>
       </c>
       <c r="F11" s="27">
-        <f t="array" ref="F11">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>4</v>
+        <f t="array" ref="F11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>9</v>
       </c>
       <c r="G11" s="12">
-        <f t="array" ref="G11">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>16</v>
+        <f t="array" ref="G11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>11</v>
       </c>
       <c r="H11" s="26">
-        <f t="array" ref="H11">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>2</v>
+        <f t="array" ref="H11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>15</v>
       </c>
       <c r="I11" s="27">
-        <f t="array" ref="I11">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>10</v>
+        <f t="array" ref="I11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>1</v>
       </c>
       <c r="J11" s="12">
-        <f t="array" ref="J11">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>12</v>
+        <f t="array" ref="J11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>5</v>
       </c>
       <c r="K11" s="26">
-        <f t="array" ref="K11">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),
-      $J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>18</v>
+        <f t="array" ref="K11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>17</v>
       </c>
       <c r="L11" s="12"/>
       <c r="O11" s="22">
@@ -1962,14 +1974,14 @@
         <v>3</v>
       </c>
       <c r="P11" s="23" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="Q11" s="24">
         <f>[1]Schedule!D17</f>
         <v>15</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="U11" s="12">
         <v>17</v>
@@ -1999,7 +2011,7 @@
         <v>1</v>
       </c>
       <c r="AD11" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="AE11" s="12">
         <v>4</v>
@@ -2029,7 +2041,7 @@
         <v>8</v>
       </c>
       <c r="AN11" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="AO11" s="12">
         <v>7</v>
@@ -2059,7 +2071,7 @@
         <v>3</v>
       </c>
       <c r="AX11" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="AY11" s="12">
         <v>14</v>
@@ -2088,58 +2100,118 @@
       <c r="BG11" s="12">
         <v>18</v>
       </c>
+      <c r="BH11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="BI11" s="12">
+        <v>7</v>
+      </c>
+      <c r="BJ11" s="12">
+        <v>3</v>
+      </c>
+      <c r="BK11" s="12">
+        <v>13</v>
+      </c>
+      <c r="BL11" s="12">
+        <v>9</v>
+      </c>
+      <c r="BM11" s="12">
+        <v>11</v>
+      </c>
+      <c r="BN11" s="12">
+        <v>15</v>
+      </c>
+      <c r="BO11" s="12">
+        <v>1</v>
+      </c>
+      <c r="BP11" s="12">
+        <v>5</v>
+      </c>
+      <c r="BQ11" s="12">
+        <v>17</v>
+      </c>
+      <c r="BR11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="BS11" s="12">
+        <v>2</v>
+      </c>
+      <c r="BT11" s="12">
+        <v>6</v>
+      </c>
+      <c r="BU11" s="12">
+        <v>12</v>
+      </c>
+      <c r="BV11" s="12">
+        <v>14</v>
+      </c>
+      <c r="BW11" s="12">
+        <v>16</v>
+      </c>
+      <c r="BX11" s="12">
+        <v>18</v>
+      </c>
+      <c r="BY11" s="12">
+        <v>8</v>
+      </c>
+      <c r="BZ11" s="12">
+        <v>4</v>
+      </c>
+      <c r="CA11" s="12">
+        <v>10</v>
+      </c>
     </row>
-    <row r="12" spans="2:59" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:79" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="28" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C12" s="29">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D12" s="30">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E12" s="31">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F12" s="29">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G12" s="30">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H12" s="31">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I12" s="29">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J12" s="30">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K12" s="31">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L12" s="12">
         <f>SUM(C12:K12)</f>
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="M12" s="32">
         <f>SUM(C12:K12)-SUM(C$10:K$10)</f>
+        <v>6</v>
+      </c>
+      <c r="O12" s="22">
+        <v>4</v>
+      </c>
+      <c r="P12" s="23" t="s">
         <v>34</v>
-      </c>
-      <c r="O12" s="22">
-        <v>4</v>
-      </c>
-      <c r="P12" s="23" t="s">
-        <v>32</v>
       </c>
       <c r="Q12" s="24">
         <f>[1]Schedule!D18</f>
         <v>20</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="U12" s="33">
         <v>4</v>
@@ -2169,7 +2241,7 @@
         <v>4</v>
       </c>
       <c r="AD12" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="AE12" s="33">
         <v>4</v>
@@ -2199,7 +2271,7 @@
         <v>5</v>
       </c>
       <c r="AN12" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="AO12" s="33">
         <v>4</v>
@@ -2229,7 +2301,7 @@
         <v>4</v>
       </c>
       <c r="AX12" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="AY12" s="33">
         <v>4</v>
@@ -2258,66 +2330,126 @@
       <c r="BG12" s="33">
         <v>5</v>
       </c>
+      <c r="BH12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="BI12" s="33">
+        <v>5</v>
+      </c>
+      <c r="BJ12" s="33">
+        <v>4</v>
+      </c>
+      <c r="BK12" s="33">
+        <v>3</v>
+      </c>
+      <c r="BL12" s="33">
+        <v>5</v>
+      </c>
+      <c r="BM12" s="33">
+        <v>4</v>
+      </c>
+      <c r="BN12" s="33">
+        <v>3</v>
+      </c>
+      <c r="BO12" s="33">
+        <v>4</v>
+      </c>
+      <c r="BP12" s="33">
+        <v>3</v>
+      </c>
+      <c r="BQ12" s="33">
+        <v>4</v>
+      </c>
+      <c r="BR12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="BS12" s="33">
+        <v>4</v>
+      </c>
+      <c r="BT12" s="33">
+        <v>4</v>
+      </c>
+      <c r="BU12" s="33">
+        <v>3</v>
+      </c>
+      <c r="BV12" s="33">
+        <v>5</v>
+      </c>
+      <c r="BW12" s="33">
+        <v>4</v>
+      </c>
+      <c r="BX12" s="33">
+        <v>4</v>
+      </c>
+      <c r="BY12" s="33">
+        <v>3</v>
+      </c>
+      <c r="BZ12" s="33">
+        <v>5</v>
+      </c>
+      <c r="CA12" s="33">
+        <v>4</v>
+      </c>
     </row>
-    <row r="13" spans="2:59" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:79" x14ac:dyDescent="0.25">
       <c r="B13" s="25" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C13" s="27">
         <f t="shared" ref="C13:K13" si="0">INT($D$8/18)+IF(C11&lt;=MOD($D$8,18),1,0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" s="12">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" s="26">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F13" s="27">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G13" s="12">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H13" s="26">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I13" s="27">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J13" s="12">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" s="26">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L13" s="32"/>
       <c r="O13" s="22">
         <v>5</v>
       </c>
       <c r="P13" s="23" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="Q13" s="24">
         <f>[1]Schedule!D19</f>
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="2:59" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:79" x14ac:dyDescent="0.25">
       <c r="B14" s="25" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C14" s="27">
         <f>C12-C13</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D14" s="12">
         <f t="shared" ref="D14:K14" si="1">D12-INT($D$8/18)-IF(D11&lt;=MOD($D$8,18),1,0)</f>
@@ -2325,23 +2457,23 @@
       </c>
       <c r="E14" s="26">
         <f t="shared" si="1"/>
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F14" s="27">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G14" s="12">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H14" s="26">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I14" s="27">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J14" s="12">
         <f t="shared" si="1"/>
@@ -2349,50 +2481,50 @@
       </c>
       <c r="K14" s="26">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L14" s="34">
         <f>SUM(C14:K14)</f>
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="M14" s="32">
         <f>SUM(C14:K14)-SUM(C$10:K$10)</f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="O14" s="22">
         <v>6</v>
       </c>
       <c r="P14" s="23" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="Q14" s="24">
         <f>[1]Schedule!D20</f>
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="2:59" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:79" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="35" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C15" s="36">
         <f t="shared" ref="C15:K15" si="2">IF(C14&lt;C23,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" s="37">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="38">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" s="36">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" s="37">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15" s="38">
         <f t="shared" si="2"/>
@@ -2404,7 +2536,7 @@
       </c>
       <c r="J15" s="37">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15" s="38">
         <f t="shared" si="2"/>
@@ -2416,14 +2548,14 @@
         <v>7</v>
       </c>
       <c r="P15" s="23" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="Q15" s="24">
         <f>[1]Schedule!D21</f>
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="2:59" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:79" x14ac:dyDescent="0.25">
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
       <c r="E16" s="12"/>
@@ -2438,38 +2570,38 @@
         <v>8</v>
       </c>
       <c r="P16" s="23" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="Q16" s="24">
         <f>[1]Schedule!D22</f>
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="2:42" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:17" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="13" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D17" s="12">
         <f>_xlfn.XLOOKUP(B17,$P$9:$P$23,$Q$9:$Q$23)</f>
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="E17" s="12"/>
       <c r="F17" s="12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H17" s="12"/>
       <c r="I17" s="12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J17" s="12" t="str">
         <f>J8</f>
-        <v>Back 9</v>
+        <v>Front 9</v>
       </c>
       <c r="K17" s="12"/>
       <c r="L17" s="12"/>
@@ -2477,16 +2609,16 @@
         <v>9</v>
       </c>
       <c r="P17" s="23" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Q17" s="24">
         <f>[1]Schedule!D23</f>
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="2:42" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="18" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C18" s="19">
         <v>1</v>
@@ -2521,269 +2653,107 @@
         <v>10</v>
       </c>
       <c r="P18" s="23" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="Q18" s="24">
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="2:42" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B19" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C19" s="12">
-        <f t="array" ref="C19">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AE$12:$AM$12,1,C18),
-      $J17="Front 9",INDEX($U$12:$AC$12,1,C18)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AY$12:$BG$12,1,C18),
-      $J17="Front 9",INDEX($AO$12:$AW$12,1,C18)
-   )
-)</f>
-        <v>4</v>
+        <f t="array" ref="C19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,C18),$J17="Front 9",INDEX($U$12:$AC$12,1,C18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,C18),$J17="Front 9",INDEX($AO$12:$AW$12,1,C18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,C18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,C18)))</f>
+        <v>5</v>
       </c>
       <c r="D19" s="12">
-        <f t="array" ref="D19">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AE$12:$AM$12,1,D18),
-      $J17="Front 9",INDEX($U$12:$AC$12,1,D18)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AY$12:$BG$12,1,D18),
-      $J17="Front 9",INDEX($AO$12:$AW$12,1,D18)
-   )
-)</f>
-        <v>3</v>
+        <f t="array" ref="D19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,D18),$J17="Front 9",INDEX($U$12:$AC$12,1,D18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,D18),$J17="Front 9",INDEX($AO$12:$AW$12,1,D18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,D18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,D18)))</f>
+        <v>4</v>
       </c>
       <c r="E19" s="26">
-        <f t="array" ref="E19">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AE$12:$AM$12,1,E18),
-      $J17="Front 9",INDEX($U$12:$AC$12,1,E18)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AY$12:$BG$12,1,E18),
-      $J17="Front 9",INDEX($AO$12:$AW$12,1,E18)
-   )
-)</f>
-        <v>5</v>
+        <f t="array" ref="E19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,E18),$J17="Front 9",INDEX($U$12:$AC$12,1,E18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,E18),$J17="Front 9",INDEX($AO$12:$AW$12,1,E18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,E18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,E18)))</f>
+        <v>3</v>
       </c>
       <c r="F19" s="27">
-        <f t="array" ref="F19">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AE$12:$AM$12,1,F18),
-      $J17="Front 9",INDEX($U$12:$AC$12,1,F18)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AY$12:$BG$12,1,F18),
-      $J17="Front 9",INDEX($AO$12:$AW$12,1,F18)
-   )
-)</f>
-        <v>4</v>
+        <f t="array" ref="F19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,F18),$J17="Front 9",INDEX($U$12:$AC$12,1,F18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,F18),$J17="Front 9",INDEX($AO$12:$AW$12,1,F18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,F18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,F18)))</f>
+        <v>5</v>
       </c>
       <c r="G19" s="12">
-        <f t="array" ref="G19">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AE$12:$AM$12,1,G18),
-      $J17="Front 9",INDEX($U$12:$AC$12,1,G18)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AY$12:$BG$12,1,G18),
-      $J17="Front 9",INDEX($AO$12:$AW$12,1,G18)
-   )
-)</f>
+        <f t="array" ref="G19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,G18),$J17="Front 9",INDEX($U$12:$AC$12,1,G18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,G18),$J17="Front 9",INDEX($AO$12:$AW$12,1,G18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,G18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,G18)))</f>
         <v>4</v>
       </c>
       <c r="H19" s="26">
-        <f t="array" ref="H19">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AE$12:$AM$12,1,H18),
-      $J17="Front 9",INDEX($U$12:$AC$12,1,H18)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AY$12:$BG$12,1,H18),
-      $J17="Front 9",INDEX($AO$12:$AW$12,1,H18)
-   )
-)</f>
-        <v>4</v>
+        <f t="array" ref="H19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,H18),$J17="Front 9",INDEX($U$12:$AC$12,1,H18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,H18),$J17="Front 9",INDEX($AO$12:$AW$12,1,H18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,H18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,H18)))</f>
+        <v>3</v>
       </c>
       <c r="I19" s="27">
-        <f t="array" ref="I19">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AE$12:$AM$12,1,I18),
-      $J17="Front 9",INDEX($U$12:$AC$12,1,I18)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AY$12:$BG$12,1,I18),
-      $J17="Front 9",INDEX($AO$12:$AW$12,1,I18)
-   )
-)</f>
+        <f t="array" ref="I19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,I18),$J17="Front 9",INDEX($U$12:$AC$12,1,I18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,I18),$J17="Front 9",INDEX($AO$12:$AW$12,1,I18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,I18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,I18)))</f>
         <v>4</v>
       </c>
       <c r="J19" s="12">
-        <f t="array" ref="J19">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AE$12:$AM$12,1,J18),
-      $J17="Front 9",INDEX($U$12:$AC$12,1,J18)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AY$12:$BG$12,1,J18),
-      $J17="Front 9",INDEX($AO$12:$AW$12,1,J18)
-   )
-)</f>
+        <f t="array" ref="J19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,J18),$J17="Front 9",INDEX($U$12:$AC$12,1,J18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,J18),$J17="Front 9",INDEX($AO$12:$AW$12,1,J18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,J18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,J18)))</f>
         <v>3</v>
       </c>
       <c r="K19" s="26">
-        <f t="array" ref="K19">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AE$12:$AM$12,1,K18),
-      $J17="Front 9",INDEX($U$12:$AC$12,1,K18)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",INDEX($AY$12:$BG$12,1,K18),
-      $J17="Front 9",INDEX($AO$12:$AW$12,1,K18)
-   )
-)</f>
-        <v>5</v>
+        <f t="array" ref="K19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,K18),$J17="Front 9",INDEX($U$12:$AC$12,1,K18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,K18),$J17="Front 9",INDEX($AO$12:$AW$12,1,K18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,K18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,K18)))</f>
+        <v>4</v>
       </c>
       <c r="L19" s="12">
         <f>SUM(C19:K19)</f>
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O19" s="22">
         <f>O18+1</f>
         <v>11</v>
       </c>
       <c r="P19" s="23" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="Q19" s="24">
         <f>[1]Schedule!D25</f>
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="2:42" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B20" s="25" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C20" s="12">
-        <f t="array" ref="C20">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>14</v>
+        <f t="array" ref="C20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>7</v>
       </c>
       <c r="D20" s="12">
-        <f t="array" ref="D20">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>8</v>
+        <f t="array" ref="D20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>3</v>
       </c>
       <c r="E20" s="26">
-        <f t="array" ref="E20">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>6</v>
+        <f t="array" ref="E20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>13</v>
       </c>
       <c r="F20" s="27">
-        <f t="array" ref="F20">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>4</v>
+        <f t="array" ref="F20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>9</v>
       </c>
       <c r="G20" s="12">
-        <f t="array" ref="G20">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>16</v>
+        <f t="array" ref="G20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>11</v>
       </c>
       <c r="H20" s="26">
-        <f t="array" ref="H20">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>2</v>
+        <f t="array" ref="H20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>15</v>
       </c>
       <c r="I20" s="27">
-        <f t="array" ref="I20">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>10</v>
+        <f t="array" ref="I20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>1</v>
       </c>
       <c r="J20" s="12">
-        <f t="array" ref="J20">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>12</v>
+        <f t="array" ref="J20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>5</v>
       </c>
       <c r="K20" s="26">
-        <f t="array" ref="K20">IF($B$2="Skybrook",
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)
-   ),
-   _xlfn.IFS(
-      $J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),
-      $J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)
-   )
-)</f>
-        <v>18</v>
+        <f t="array" ref="K20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
+        <v>17</v>
       </c>
       <c r="L20" s="12"/>
       <c r="O20" s="22">
@@ -2797,63 +2767,63 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="2:42" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="28" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C21" s="29">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D21" s="30">
+        <v>7</v>
+      </c>
+      <c r="E21" s="31">
         <v>6</v>
-      </c>
-      <c r="E21" s="31">
-        <v>10</v>
       </c>
       <c r="F21" s="29">
         <v>8</v>
       </c>
       <c r="G21" s="30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H21" s="31">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I21" s="29">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J21" s="30">
         <v>6</v>
       </c>
       <c r="K21" s="31">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L21" s="12">
         <f>SUM(C21:K21)</f>
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="M21" s="32">
         <f>SUM(C21:K21)-SUM(C$10:K$10)</f>
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="O21" s="22">
         <v>13</v>
       </c>
       <c r="P21" s="23" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="Q21" s="24">
         <f>[1]Schedule!D27</f>
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="2:42" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B22" s="25" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C22" s="27">
         <f t="shared" ref="C22:K22" si="3">INT($D$17/18)+IF(C20&lt;=MOD($D$17,18),1,0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" s="12">
         <f t="shared" si="3"/>
@@ -2861,19 +2831,19 @@
       </c>
       <c r="E22" s="26">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" s="27">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G22" s="12">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H22" s="26">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I22" s="27">
         <f t="shared" si="3"/>
@@ -2881,59 +2851,59 @@
       </c>
       <c r="J22" s="12">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K22" s="26">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L22" s="32"/>
       <c r="O22" s="22">
         <v>14</v>
       </c>
       <c r="P22" s="23" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="Q22" s="24">
         <f>[1]Schedule!D28</f>
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="2:42" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B23" s="25" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C23" s="27">
         <f t="shared" ref="C23:K23" si="4">C21-C22</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D23" s="12">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E23" s="26">
         <f t="shared" si="4"/>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F23" s="27">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G23" s="12">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H23" s="26">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I23" s="27">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J23" s="12">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K23" s="26">
         <f t="shared" si="4"/>
@@ -2941,26 +2911,26 @@
       </c>
       <c r="L23" s="34">
         <f>SUM(C23:K23)</f>
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="M23" s="32">
         <f>SUM(C23:K23)-SUM(C$10:K$10)</f>
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="O23" s="22">
         <v>15</v>
       </c>
       <c r="P23" s="23" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="Q23" s="24">
         <f>[1]Schedule!D29</f>
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="2:42" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:17" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B24" s="35" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C24" s="36">
         <f t="shared" ref="C24:K24" si="5">IF(C23&lt;C14,1,0)</f>
@@ -2980,11 +2950,11 @@
       </c>
       <c r="G24" s="37">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H24" s="38">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" s="36">
         <f t="shared" si="5"/>
@@ -3000,26 +2970,24 @@
       </c>
       <c r="L24" s="12"/>
     </row>
-    <row r="29" spans="2:42" x14ac:dyDescent="0.2">
-      <c r="AP29" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="16">
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="T7:AM7"/>
     <mergeCell ref="J1:M1"/>
+    <mergeCell ref="AD8:AM8"/>
+    <mergeCell ref="AX8:BG8"/>
+    <mergeCell ref="AN7:BG7"/>
+    <mergeCell ref="L3:M5"/>
+    <mergeCell ref="U8:AC8"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="AO8:AW8"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="BH7:CA7"/>
+    <mergeCell ref="J3:K5"/>
     <mergeCell ref="J2:K2"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="J3:K5"/>
-    <mergeCell ref="L3:M5"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="T7:AM7"/>
-    <mergeCell ref="AN7:BG7"/>
-    <mergeCell ref="U8:AC8"/>
-    <mergeCell ref="AD8:AM8"/>
-    <mergeCell ref="AO8:AW8"/>
-    <mergeCell ref="AX8:BG8"/>
+    <mergeCell ref="BR8:CA8"/>
+    <mergeCell ref="BI8:BQ8"/>
   </mergeCells>
   <conditionalFormatting sqref="C15:K15 C24:K24">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
@@ -3027,16 +2995,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8 B17" xr:uid="{C9AEDD85-A7D3-4E4C-B668-7AD01D2A0F97}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8 B17" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$P$9:$P$23</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G8 G17 G29" xr:uid="{99534488-80E5-4A0C-85E7-5CBC12771C2B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G8 G17 G29" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>INDIRECT(SUBSTITUTE($B$2," ","_"))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{09069BF6-4B93-4325-A190-3182B6A4A52F}">
-      <formula1>$T$7:$BG$7</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{00000000-0002-0000-0000-000002000000}">
+      <formula1>$T$7:$CA$7</formula1>
     </dataValidation>
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="J8 J17" xr:uid="{98653412-F62B-4706-828B-0A2A536F6752}">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="J8 J17" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>$U$8:$AD$8</formula1>
     </dataValidation>
   </dataValidations>
@@ -3045,44 +3013,56 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9023B9F3-7138-4C94-97BC-0498273A3425}">
-  <dimension ref="C2:D5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="C2:E5"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C2" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>46</v>
+        <v>49</v>
+      </c>
+      <c r="E2" t="s">
+        <v>50</v>
       </c>
     </row>
-    <row r="3" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="4" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>29</v>
+      </c>
+      <c r="E4" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="5" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>30</v>
+        <v>32</v>
+      </c>
+      <c r="E5" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Scores: R4 Michael def. Brian 4.5-3.5; Carson def. Ethan 5-3 (Bruce-replacement pickup); HC adjust Carson->24, Michael->25
- R4 @ Warrior: Michael McHugh 4.5 (NET 40) def. Brian Wojcio 3.5 (NET 39) -> Michael 2-2-0, Brian 1-2-1
- R4 @ Warrior: Carson Bass 5 (NET 34) def. Ethan High 3 (NET 38) -> Carson's Bruce-replacement pickup; Carson 2-2-0
- Pickup/drop-lowest: Ethan's 3-pt pickup loss is his lowest round, dropped per mulligan rule; Ethan unchanged at 27 pts, 4-0-0 (R4 counting result remains def. Alex Palmer 7-1)
- Handicaps revised effective R4 onward: Carson Bass 20->24, Michael McHugh 22->25 (master Schedule tab); R1-R3 stand as played
- Standings: Brian #6, Carson up to #7 (2-2-0), Michael #9 (2-2-0)
- R4 now 6 of 7 (outstanding: Rob Bass vs Curtis Lynn)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Score Calculator.xlsx
+++ b/Score Calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imicompanies-my.sharepoint.com/personal/ehigh_iengtobuild_com/Documents/Documents/Golf League/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="11_D812028DA688F3B9538958C5B423B5CF7585794A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DDAEABDB-36BE-4790-90A7-DB2C3E8BE5E5}"/>
+  <xr:revisionPtr revIDLastSave="90" documentId="11_D812028DA688F3B9538958C5B423B5CF7585794A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A619D9F8-11CF-4C4F-BE4A-2466B3DA75C5}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculator" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,6 @@
     <definedName name="Warrior_Golf_Club">Helper!$E$3:$E$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -586,12 +585,26 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -599,23 +612,9 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -649,6 +648,9 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Scores 2024"/>
       <sheetName val="Sep 2 - 13th"/>
@@ -689,12 +691,12 @@
         </row>
         <row r="18">
           <cell r="D18">
-            <v>20</v>
+            <v>24</v>
           </cell>
         </row>
         <row r="19">
           <cell r="D19">
-            <v>22</v>
+            <v>25</v>
           </cell>
         </row>
         <row r="20">
@@ -715,6 +717,11 @@
         <row r="23">
           <cell r="D23">
             <v>28</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="D24">
+            <v>20</v>
           </cell>
         </row>
         <row r="25">
@@ -1107,12 +1114,12 @@
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J1" s="51" t="s">
-        <v>1</v>
-      </c>
-      <c r="K1" s="52"/>
-      <c r="L1" s="52"/>
-      <c r="M1" s="52"/>
+      <c r="J1" s="43" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
+      <c r="M1" s="44"/>
     </row>
     <row r="2" spans="2:79" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
@@ -1134,28 +1141,28 @@
         <v>7</v>
       </c>
       <c r="I2" s="5"/>
-      <c r="J2" s="49" t="str">
+      <c r="J2" s="53" t="str">
         <f>B8</f>
+        <v>Ethan High</v>
+      </c>
+      <c r="K2" s="50"/>
+      <c r="L2" s="49" t="str">
+        <f>B17</f>
         <v>Carson Bass</v>
       </c>
-      <c r="K2" s="42"/>
-      <c r="L2" s="41" t="str">
-        <f>B17</f>
-        <v>Brian Wojcio</v>
-      </c>
-      <c r="M2" s="42"/>
+      <c r="M2" s="50"/>
     </row>
     <row r="3" spans="2:79" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="50" t="str">
+      <c r="B3" s="39" t="str">
         <f>J2</f>
-        <v>Carson Bass</v>
+        <v>Ethan High</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="7">
         <f>SUM(C15:E15)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" s="7">
         <f>SUM(F15:H15)</f>
@@ -1167,31 +1174,31 @@
       </c>
       <c r="G3" s="7">
         <f>SUM(C15:K15)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3" s="7">
         <f>SUM(C14:K14)</f>
-        <v>47</v>
-      </c>
-      <c r="J3" s="43">
+        <v>38</v>
+      </c>
+      <c r="J3" s="51">
         <f>SUM(D4:H4)</f>
-        <v>0</v>
-      </c>
-      <c r="K3" s="44"/>
-      <c r="L3" s="53">
+        <v>3</v>
+      </c>
+      <c r="K3" s="46"/>
+      <c r="L3" s="45">
         <f>SUM(D6:H6)</f>
-        <v>8</v>
-      </c>
-      <c r="M3" s="44"/>
+        <v>5</v>
+      </c>
+      <c r="M3" s="46"/>
     </row>
     <row r="4" spans="2:79" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="47"/>
+      <c r="B4" s="40"/>
       <c r="C4" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="9">
         <f>IF(D3&gt;D5,2,IF(D3=D5,1,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="9">
         <f>IF(E3&gt;E5,2,IF(E3=E5,1,0))</f>
@@ -1199,7 +1206,7 @@
       </c>
       <c r="F4" s="9">
         <f>IF(F3&gt;F5,2,IF(F3=F5,1,0))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G4" s="9">
         <f>IF(G3&gt;G5,1,IF(G3=G5,0.5,0))</f>
@@ -1209,22 +1216,22 @@
         <f>IF(H3&lt;H5,1,IF(H3=H5,0.5,0))</f>
         <v>0</v>
       </c>
-      <c r="J4" s="45"/>
-      <c r="K4" s="46"/>
-      <c r="L4" s="40"/>
-      <c r="M4" s="46"/>
+      <c r="J4" s="52"/>
+      <c r="K4" s="47"/>
+      <c r="L4" s="42"/>
+      <c r="M4" s="47"/>
     </row>
     <row r="5" spans="2:79" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="50" t="str">
+      <c r="B5" s="39" t="str">
         <f>L2</f>
-        <v>Brian Wojcio</v>
+        <v>Carson Bass</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="11">
         <f>SUM(C24:E24)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E5" s="11">
         <f>SUM(F24:H24)</f>
@@ -1232,29 +1239,29 @@
       </c>
       <c r="F5" s="11">
         <f>SUM(I24:K24)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5" s="11">
         <f>SUM(C24:K24)</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H5" s="11">
         <f>SUM(C23:K23)</f>
         <v>34</v>
       </c>
-      <c r="J5" s="47"/>
+      <c r="J5" s="40"/>
       <c r="K5" s="48"/>
-      <c r="L5" s="52"/>
+      <c r="L5" s="44"/>
       <c r="M5" s="48"/>
     </row>
     <row r="6" spans="2:79" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="47"/>
+      <c r="B6" s="40"/>
       <c r="C6" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D6" s="9">
         <f>IF(D5&gt;D3,2,IF(D5=D3,1,0))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" s="9">
         <f>IF(E5&gt;E3,2,IF(E5=E3,1,0))</f>
@@ -1262,7 +1269,7 @@
       </c>
       <c r="F6" s="9">
         <f>IF(F5&gt;F3,2,IF(F5=F3,1,0))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G6" s="9">
         <f>IF(G5&gt;G3,1,IF(G5=G3,0.5,0))</f>
@@ -1288,83 +1295,83 @@
       <c r="J7" s="12"/>
       <c r="K7" s="12"/>
       <c r="L7" s="12"/>
-      <c r="T7" s="39" t="s">
+      <c r="T7" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="U7" s="40"/>
-      <c r="V7" s="40"/>
-      <c r="W7" s="40"/>
-      <c r="X7" s="40"/>
-      <c r="Y7" s="40"/>
-      <c r="Z7" s="40"/>
-      <c r="AA7" s="40"/>
-      <c r="AB7" s="40"/>
-      <c r="AC7" s="40"/>
-      <c r="AD7" s="40"/>
-      <c r="AE7" s="40"/>
-      <c r="AF7" s="40"/>
-      <c r="AG7" s="40"/>
-      <c r="AH7" s="40"/>
-      <c r="AI7" s="40"/>
-      <c r="AJ7" s="40"/>
-      <c r="AK7" s="40"/>
-      <c r="AL7" s="40"/>
-      <c r="AM7" s="40"/>
-      <c r="AN7" s="39" t="s">
+      <c r="U7" s="42"/>
+      <c r="V7" s="42"/>
+      <c r="W7" s="42"/>
+      <c r="X7" s="42"/>
+      <c r="Y7" s="42"/>
+      <c r="Z7" s="42"/>
+      <c r="AA7" s="42"/>
+      <c r="AB7" s="42"/>
+      <c r="AC7" s="42"/>
+      <c r="AD7" s="42"/>
+      <c r="AE7" s="42"/>
+      <c r="AF7" s="42"/>
+      <c r="AG7" s="42"/>
+      <c r="AH7" s="42"/>
+      <c r="AI7" s="42"/>
+      <c r="AJ7" s="42"/>
+      <c r="AK7" s="42"/>
+      <c r="AL7" s="42"/>
+      <c r="AM7" s="42"/>
+      <c r="AN7" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="AO7" s="40"/>
-      <c r="AP7" s="40"/>
-      <c r="AQ7" s="40"/>
-      <c r="AR7" s="40"/>
-      <c r="AS7" s="40"/>
-      <c r="AT7" s="40"/>
-      <c r="AU7" s="40"/>
-      <c r="AV7" s="40"/>
-      <c r="AW7" s="40"/>
-      <c r="AX7" s="40"/>
-      <c r="AY7" s="40"/>
-      <c r="AZ7" s="40"/>
-      <c r="BA7" s="40"/>
-      <c r="BB7" s="40"/>
-      <c r="BC7" s="40"/>
-      <c r="BD7" s="40"/>
-      <c r="BE7" s="40"/>
-      <c r="BF7" s="40"/>
-      <c r="BG7" s="40"/>
-      <c r="BH7" s="39" t="s">
+      <c r="AO7" s="42"/>
+      <c r="AP7" s="42"/>
+      <c r="AQ7" s="42"/>
+      <c r="AR7" s="42"/>
+      <c r="AS7" s="42"/>
+      <c r="AT7" s="42"/>
+      <c r="AU7" s="42"/>
+      <c r="AV7" s="42"/>
+      <c r="AW7" s="42"/>
+      <c r="AX7" s="42"/>
+      <c r="AY7" s="42"/>
+      <c r="AZ7" s="42"/>
+      <c r="BA7" s="42"/>
+      <c r="BB7" s="42"/>
+      <c r="BC7" s="42"/>
+      <c r="BD7" s="42"/>
+      <c r="BE7" s="42"/>
+      <c r="BF7" s="42"/>
+      <c r="BG7" s="42"/>
+      <c r="BH7" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="BI7" s="40"/>
-      <c r="BJ7" s="40"/>
-      <c r="BK7" s="40"/>
-      <c r="BL7" s="40"/>
-      <c r="BM7" s="40"/>
-      <c r="BN7" s="40"/>
-      <c r="BO7" s="40"/>
-      <c r="BP7" s="40"/>
-      <c r="BQ7" s="40"/>
-      <c r="BR7" s="40"/>
-      <c r="BS7" s="40"/>
-      <c r="BT7" s="40"/>
-      <c r="BU7" s="40"/>
-      <c r="BV7" s="40"/>
-      <c r="BW7" s="40"/>
-      <c r="BX7" s="40"/>
-      <c r="BY7" s="40"/>
-      <c r="BZ7" s="40"/>
-      <c r="CA7" s="40"/>
+      <c r="BI7" s="42"/>
+      <c r="BJ7" s="42"/>
+      <c r="BK7" s="42"/>
+      <c r="BL7" s="42"/>
+      <c r="BM7" s="42"/>
+      <c r="BN7" s="42"/>
+      <c r="BO7" s="42"/>
+      <c r="BP7" s="42"/>
+      <c r="BQ7" s="42"/>
+      <c r="BR7" s="42"/>
+      <c r="BS7" s="42"/>
+      <c r="BT7" s="42"/>
+      <c r="BU7" s="42"/>
+      <c r="BV7" s="42"/>
+      <c r="BW7" s="42"/>
+      <c r="BX7" s="42"/>
+      <c r="BY7" s="42"/>
+      <c r="BZ7" s="42"/>
+      <c r="CA7" s="42"/>
     </row>
     <row r="8" spans="2:79" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="13" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C8" s="14" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="12">
         <f>_xlfn.XLOOKUP(B8,$P$9:$P$23,$Q$9:$Q$23)</f>
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="12" t="s">
@@ -1378,7 +1385,7 @@
         <v>16</v>
       </c>
       <c r="J8" s="16" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="K8" s="12"/>
       <c r="L8" s="12"/>
@@ -1394,81 +1401,81 @@
       <c r="T8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="U8" s="39" t="s">
+      <c r="U8" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="V8" s="40"/>
-      <c r="W8" s="40"/>
-      <c r="X8" s="40"/>
-      <c r="Y8" s="40"/>
-      <c r="Z8" s="40"/>
-      <c r="AA8" s="40"/>
-      <c r="AB8" s="40"/>
-      <c r="AC8" s="40"/>
-      <c r="AD8" s="39" t="s">
+      <c r="V8" s="42"/>
+      <c r="W8" s="42"/>
+      <c r="X8" s="42"/>
+      <c r="Y8" s="42"/>
+      <c r="Z8" s="42"/>
+      <c r="AA8" s="42"/>
+      <c r="AB8" s="42"/>
+      <c r="AC8" s="42"/>
+      <c r="AD8" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="AE8" s="40"/>
-      <c r="AF8" s="40"/>
-      <c r="AG8" s="40"/>
-      <c r="AH8" s="40"/>
-      <c r="AI8" s="40"/>
-      <c r="AJ8" s="40"/>
-      <c r="AK8" s="40"/>
-      <c r="AL8" s="40"/>
-      <c r="AM8" s="40"/>
+      <c r="AE8" s="42"/>
+      <c r="AF8" s="42"/>
+      <c r="AG8" s="42"/>
+      <c r="AH8" s="42"/>
+      <c r="AI8" s="42"/>
+      <c r="AJ8" s="42"/>
+      <c r="AK8" s="42"/>
+      <c r="AL8" s="42"/>
+      <c r="AM8" s="42"/>
       <c r="AN8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="AO8" s="39" t="s">
+      <c r="AO8" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="AP8" s="40"/>
-      <c r="AQ8" s="40"/>
-      <c r="AR8" s="40"/>
-      <c r="AS8" s="40"/>
-      <c r="AT8" s="40"/>
-      <c r="AU8" s="40"/>
-      <c r="AV8" s="40"/>
-      <c r="AW8" s="40"/>
-      <c r="AX8" s="39" t="s">
+      <c r="AP8" s="42"/>
+      <c r="AQ8" s="42"/>
+      <c r="AR8" s="42"/>
+      <c r="AS8" s="42"/>
+      <c r="AT8" s="42"/>
+      <c r="AU8" s="42"/>
+      <c r="AV8" s="42"/>
+      <c r="AW8" s="42"/>
+      <c r="AX8" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="AY8" s="40"/>
-      <c r="AZ8" s="40"/>
-      <c r="BA8" s="40"/>
-      <c r="BB8" s="40"/>
-      <c r="BC8" s="40"/>
-      <c r="BD8" s="40"/>
-      <c r="BE8" s="40"/>
-      <c r="BF8" s="40"/>
-      <c r="BG8" s="40"/>
+      <c r="AY8" s="42"/>
+      <c r="AZ8" s="42"/>
+      <c r="BA8" s="42"/>
+      <c r="BB8" s="42"/>
+      <c r="BC8" s="42"/>
+      <c r="BD8" s="42"/>
+      <c r="BE8" s="42"/>
+      <c r="BF8" s="42"/>
+      <c r="BG8" s="42"/>
       <c r="BH8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="BI8" s="39" t="s">
+      <c r="BI8" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="BJ8" s="40"/>
-      <c r="BK8" s="40"/>
-      <c r="BL8" s="40"/>
-      <c r="BM8" s="40"/>
-      <c r="BN8" s="40"/>
-      <c r="BO8" s="40"/>
-      <c r="BP8" s="40"/>
-      <c r="BQ8" s="40"/>
-      <c r="BR8" s="39" t="s">
+      <c r="BJ8" s="42"/>
+      <c r="BK8" s="42"/>
+      <c r="BL8" s="42"/>
+      <c r="BM8" s="42"/>
+      <c r="BN8" s="42"/>
+      <c r="BO8" s="42"/>
+      <c r="BP8" s="42"/>
+      <c r="BQ8" s="42"/>
+      <c r="BR8" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="BS8" s="40"/>
-      <c r="BT8" s="40"/>
-      <c r="BU8" s="40"/>
-      <c r="BV8" s="40"/>
-      <c r="BW8" s="40"/>
-      <c r="BX8" s="40"/>
-      <c r="BY8" s="40"/>
-      <c r="BZ8" s="40"/>
-      <c r="CA8" s="40"/>
+      <c r="BS8" s="42"/>
+      <c r="BT8" s="42"/>
+      <c r="BU8" s="42"/>
+      <c r="BV8" s="42"/>
+      <c r="BW8" s="42"/>
+      <c r="BX8" s="42"/>
+      <c r="BY8" s="42"/>
+      <c r="BZ8" s="42"/>
+      <c r="CA8" s="42"/>
     </row>
     <row r="9" spans="2:79" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="18" t="s">
@@ -1699,7 +1706,7 @@
       </c>
       <c r="C10" s="12">
         <f t="array" ref="C10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,C9),$J8="Front 9",INDEX($U$12:$AC$12,1,C9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,C9),$J8="Front 9",INDEX($AO$12:$AW$12,1,C9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,C9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,C9)))</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D10" s="12">
         <f t="array" ref="D10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,D9),$J8="Front 9",INDEX($U$12:$AC$12,1,D9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,D9),$J8="Front 9",INDEX($AO$12:$AW$12,1,D9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,D9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,D9)))</f>
@@ -1719,15 +1726,15 @@
       </c>
       <c r="H10" s="26">
         <f t="array" ref="H10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,H9),$J8="Front 9",INDEX($U$12:$AC$12,1,H9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,H9),$J8="Front 9",INDEX($AO$12:$AW$12,1,H9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,H9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,H9)))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I10" s="27">
         <f t="array" ref="I10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,I9),$J8="Front 9",INDEX($U$12:$AC$12,1,I9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,I9),$J8="Front 9",INDEX($AO$12:$AW$12,1,I9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,I9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,I9)))</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J10" s="12">
         <f t="array" ref="J10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,J9),$J8="Front 9",INDEX($U$12:$AC$12,1,J9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,J9),$J8="Front 9",INDEX($AO$12:$AW$12,1,J9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,J9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,J9)))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K10" s="26">
         <f t="array" ref="K10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,K9),$J8="Front 9",INDEX($U$12:$AC$12,1,K9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,K9),$J8="Front 9",INDEX($AO$12:$AW$12,1,K9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,K9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,K9)))</f>
@@ -1735,7 +1742,7 @@
       </c>
       <c r="L10" s="12">
         <f>SUM(C10:K10)</f>
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O10" s="22">
         <v>2</v>
@@ -1934,39 +1941,39 @@
       </c>
       <c r="C11" s="12">
         <f t="array" ref="C11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D11" s="12">
         <f t="array" ref="D11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E11" s="26">
         <f t="array" ref="E11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F11" s="27">
         <f t="array" ref="F11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="G11" s="12">
         <f t="array" ref="G11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H11" s="26">
         <f t="array" ref="H11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I11" s="27">
         <f t="array" ref="I11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J11" s="12">
         <f t="array" ref="J11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K11" s="26">
         <f t="array" ref="K11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="L11" s="12"/>
       <c r="O11" s="22">
@@ -2166,39 +2173,39 @@
         <v>33</v>
       </c>
       <c r="C12" s="29">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D12" s="30">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E12" s="31">
         <v>5</v>
       </c>
       <c r="F12" s="29">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G12" s="30">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H12" s="31">
         <v>6</v>
       </c>
       <c r="I12" s="29">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J12" s="30">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K12" s="31">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L12" s="12">
         <f>SUM(C12:K12)</f>
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="M12" s="32">
         <f>SUM(C12:K12)-SUM(C$10:K$10)</f>
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="O12" s="22">
         <v>4</v>
@@ -2208,7 +2215,7 @@
       </c>
       <c r="Q12" s="24">
         <f>[1]Schedule!D18</f>
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="T12" s="2" t="s">
         <v>35</v>
@@ -2409,19 +2416,19 @@
       </c>
       <c r="F13" s="27">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" s="12">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" s="26">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="27">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J13" s="12">
         <f t="shared" si="0"/>
@@ -2440,7 +2447,7 @@
       </c>
       <c r="Q13" s="24">
         <f>[1]Schedule!D19</f>
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="2:79" x14ac:dyDescent="0.25">
@@ -2449,11 +2456,11 @@
       </c>
       <c r="C14" s="27">
         <f>C12-C13</f>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D14" s="12">
         <f t="shared" ref="D14:K14" si="1">D12-INT($D$8/18)-IF(D11&lt;=MOD($D$8,18),1,0)</f>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E14" s="26">
         <f t="shared" si="1"/>
@@ -2469,27 +2476,27 @@
       </c>
       <c r="H14" s="26">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I14" s="27">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J14" s="12">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K14" s="26">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L14" s="34">
         <f>SUM(C14:K14)</f>
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="M14" s="32">
         <f>SUM(C14:K14)-SUM(C$10:K$10)</f>
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="O14" s="22">
         <v>6</v>
@@ -2512,7 +2519,7 @@
       </c>
       <c r="D15" s="37">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="38">
         <f t="shared" si="2"/>
@@ -2536,11 +2543,11 @@
       </c>
       <c r="J15" s="37">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" s="38">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" s="12"/>
       <c r="O15" s="22">
@@ -2579,14 +2586,14 @@
     </row>
     <row r="17" spans="2:17" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="13" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C17" s="14" t="s">
         <v>13</v>
       </c>
       <c r="D17" s="12">
         <f>_xlfn.XLOOKUP(B17,$P$9:$P$23,$Q$9:$Q$23)</f>
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E17" s="12"/>
       <c r="F17" s="12" t="s">
@@ -2601,7 +2608,7 @@
       </c>
       <c r="J17" s="12" t="str">
         <f>J8</f>
-        <v>Front 9</v>
+        <v>Back 9</v>
       </c>
       <c r="K17" s="12"/>
       <c r="L17" s="12"/>
@@ -2656,6 +2663,7 @@
         <v>45</v>
       </c>
       <c r="Q18" s="24">
+        <f>[1]Schedule!D24</f>
         <v>20</v>
       </c>
     </row>
@@ -2665,7 +2673,7 @@
       </c>
       <c r="C19" s="12">
         <f t="array" ref="C19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,C18),$J17="Front 9",INDEX($U$12:$AC$12,1,C18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,C18),$J17="Front 9",INDEX($AO$12:$AW$12,1,C18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,C18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,C18)))</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D19" s="12">
         <f t="array" ref="D19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,D18),$J17="Front 9",INDEX($U$12:$AC$12,1,D18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,D18),$J17="Front 9",INDEX($AO$12:$AW$12,1,D18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,D18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,D18)))</f>
@@ -2685,15 +2693,15 @@
       </c>
       <c r="H19" s="26">
         <f t="array" ref="H19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,H18),$J17="Front 9",INDEX($U$12:$AC$12,1,H18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,H18),$J17="Front 9",INDEX($AO$12:$AW$12,1,H18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,H18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,H18)))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I19" s="27">
         <f t="array" ref="I19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,I18),$J17="Front 9",INDEX($U$12:$AC$12,1,I18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,I18),$J17="Front 9",INDEX($AO$12:$AW$12,1,I18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,I18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,I18)))</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J19" s="12">
         <f t="array" ref="J19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,J18),$J17="Front 9",INDEX($U$12:$AC$12,1,J18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,J18),$J17="Front 9",INDEX($AO$12:$AW$12,1,J18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,J18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,J18)))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K19" s="26">
         <f t="array" ref="K19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,K18),$J17="Front 9",INDEX($U$12:$AC$12,1,K18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,K18),$J17="Front 9",INDEX($AO$12:$AW$12,1,K18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,K18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,K18)))</f>
@@ -2701,7 +2709,7 @@
       </c>
       <c r="L19" s="12">
         <f>SUM(C19:K19)</f>
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O19" s="22">
         <f>O18+1</f>
@@ -2721,39 +2729,39 @@
       </c>
       <c r="C20" s="12">
         <f t="array" ref="C20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D20" s="12">
         <f t="array" ref="D20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E20" s="26">
         <f t="array" ref="E20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F20" s="27">
         <f t="array" ref="F20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="G20" s="12">
         <f t="array" ref="G20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H20" s="26">
         <f t="array" ref="H20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I20" s="27">
         <f t="array" ref="I20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J20" s="12">
         <f t="array" ref="J20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K20" s="26">
         <f t="array" ref="K20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)))</f>
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="L20" s="12"/>
       <c r="O20" s="22">
@@ -2772,39 +2780,39 @@
         <v>33</v>
       </c>
       <c r="C21" s="29">
+        <v>5</v>
+      </c>
+      <c r="D21" s="30">
         <v>6</v>
       </c>
-      <c r="D21" s="30">
-        <v>5</v>
-      </c>
       <c r="E21" s="31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F21" s="29">
         <v>5</v>
       </c>
       <c r="G21" s="30">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H21" s="31">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I21" s="29">
+        <v>4</v>
+      </c>
+      <c r="J21" s="30">
+        <v>7</v>
+      </c>
+      <c r="K21" s="31">
         <v>6</v>
-      </c>
-      <c r="J21" s="30">
-        <v>4</v>
-      </c>
-      <c r="K21" s="31">
-        <v>4</v>
       </c>
       <c r="L21" s="12">
         <f>SUM(C21:K21)</f>
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="M21" s="32">
         <f>SUM(C21:K21)-SUM(C$10:K$10)</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="O21" s="22">
         <v>13</v>
@@ -2823,15 +2831,15 @@
       </c>
       <c r="C22" s="27">
         <f t="shared" ref="C22:K22" si="3">INT($D$17/18)+IF(C20&lt;=MOD($D$17,18),1,0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" s="12">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" s="27">
         <f t="shared" si="3"/>
@@ -2843,7 +2851,7 @@
       </c>
       <c r="H22" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I22" s="27">
         <f t="shared" si="3"/>
@@ -2851,11 +2859,11 @@
       </c>
       <c r="J22" s="12">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K22" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L22" s="32"/>
       <c r="O22" s="22">
@@ -2875,7 +2883,7 @@
       </c>
       <c r="C23" s="27">
         <f t="shared" ref="C23:K23" si="4">C21-C22</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D23" s="12">
         <f t="shared" si="4"/>
@@ -2891,23 +2899,23 @@
       </c>
       <c r="G23" s="12">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H23" s="26">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I23" s="27">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J23" s="12">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K23" s="26">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L23" s="34">
         <f>SUM(C23:K23)</f>
@@ -2915,7 +2923,7 @@
       </c>
       <c r="M23" s="32">
         <f>SUM(C23:K23)-SUM(C$10:K$10)</f>
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="O23" s="22">
         <v>15</v>
@@ -2934,11 +2942,11 @@
       </c>
       <c r="C24" s="36">
         <f t="shared" ref="C24:K24" si="5">IF(C23&lt;C14,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D24" s="37">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E24" s="38">
         <f t="shared" si="5"/>
@@ -2958,7 +2966,7 @@
       </c>
       <c r="I24" s="36">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" s="37">
         <f t="shared" si="5"/>
@@ -2966,12 +2974,17 @@
       </c>
       <c r="K24" s="38">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L24" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="BH7:CA7"/>
+    <mergeCell ref="J3:K5"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="BR8:CA8"/>
+    <mergeCell ref="BI8:BQ8"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="T7:AM7"/>
     <mergeCell ref="J1:M1"/>
@@ -2983,11 +2996,6 @@
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="AO8:AW8"/>
     <mergeCell ref="L2:M2"/>
-    <mergeCell ref="BH7:CA7"/>
-    <mergeCell ref="J3:K5"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="BR8:CA8"/>
-    <mergeCell ref="BI8:BQ8"/>
   </mergeCells>
   <conditionalFormatting sqref="C15:K15 C24:K24">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">

</xml_diff>